<commit_message>
Update fuel cost workbook
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4732" uniqueCount="1768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4716" uniqueCount="1767">
   <si>
     <t xml:space="preserve">유류비 계산(혼유, 지역화폐 등)</t>
   </si>
@@ -5382,9 +5382,6 @@
   </si>
   <si>
     <t>현행화 일자: 2026-07-27</t>
-  </si>
-  <si>
-    <t>가격변동</t>
   </si>
 </sst>
 </file>
@@ -75858,164 +75855,64 @@
       </c>
     </row>
     <row r="4" s="20" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>457</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>458</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>1767</v>
-      </c>
-      <c r="E4" s="27">
-        <v>1875</v>
-      </c>
-      <c r="F4" s="27">
-        <v>1875</v>
-      </c>
-      <c r="G4" s="27">
-        <f>IF(OR(E4="",F4=""),"",F4-E4)</f>
-        <v>0</v>
-      </c>
+      <c r="A4" s="25"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
       <c r="H4" s="27"/>
       <c r="I4" s="27"/>
-      <c r="J4" s="27" t="str">
-        <f>IF(OR(H4="",I4=""),"",I4-H4)</f>
-        <v/>
-      </c>
-      <c r="K4" s="27">
-        <v>1860</v>
-      </c>
-      <c r="L4" s="27">
-        <v>1855</v>
-      </c>
-      <c r="M4" s="27">
-        <f>IF(OR(K4="",L4=""),"",L4-K4)</f>
-        <v>-5</v>
-      </c>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
     </row>
     <row r="5" s="20" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>1221</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>1222</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>1767</v>
-      </c>
-      <c r="E5" s="27">
-        <v>1844</v>
-      </c>
-      <c r="F5" s="27">
-        <v>1844</v>
-      </c>
-      <c r="G5" s="27">
-        <f>IF(OR(E5="",F5=""),"",F5-E5)</f>
-        <v>0</v>
-      </c>
+      <c r="A5" s="25"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
       <c r="H5" s="27"/>
       <c r="I5" s="27"/>
-      <c r="J5" s="27" t="str">
-        <f>IF(OR(H5="",I5=""),"",I5-H5)</f>
-        <v/>
-      </c>
-      <c r="K5" s="27">
-        <v>1834</v>
-      </c>
-      <c r="L5" s="27">
-        <v>1814</v>
-      </c>
-      <c r="M5" s="27">
-        <f>IF(OR(K5="",L5=""),"",L5-K5)</f>
-        <v>-20</v>
-      </c>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
     </row>
     <row r="6" s="20" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>1319</v>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>1320</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>1767</v>
-      </c>
-      <c r="E6" s="27">
-        <v>1850</v>
-      </c>
-      <c r="F6" s="27">
-        <v>1850</v>
-      </c>
-      <c r="G6" s="27">
-        <f>IF(OR(E6="",F6=""),"",F6-E6)</f>
-        <v>0</v>
-      </c>
+      <c r="A6" s="25"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
       <c r="H6" s="27"/>
       <c r="I6" s="27"/>
-      <c r="J6" s="27" t="str">
-        <f>IF(OR(H6="",I6=""),"",I6-H6)</f>
-        <v/>
-      </c>
-      <c r="K6" s="27">
-        <v>1810</v>
-      </c>
-      <c r="L6" s="27">
-        <v>1790</v>
-      </c>
-      <c r="M6" s="27">
-        <f>IF(OR(K6="",L6=""),"",L6-K6)</f>
-        <v>-20</v>
-      </c>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
     </row>
     <row r="7" s="20" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>1741</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>1742</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>1767</v>
-      </c>
-      <c r="E7" s="27">
-        <v>1997</v>
-      </c>
-      <c r="F7" s="27">
-        <v>1949</v>
-      </c>
-      <c r="G7" s="27">
-        <f>IF(OR(E7="",F7=""),"",F7-E7)</f>
-        <v>-48</v>
-      </c>
+      <c r="A7" s="25"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
       <c r="H7" s="27"/>
       <c r="I7" s="27"/>
-      <c r="J7" s="27" t="str">
-        <f>IF(OR(H7="",I7=""),"",I7-H7)</f>
-        <v/>
-      </c>
-      <c r="K7" s="27">
-        <v>1976</v>
-      </c>
-      <c r="L7" s="27">
-        <v>1929</v>
-      </c>
-      <c r="M7" s="27">
-        <f>IF(OR(K7="",L7=""),"",L7-K7)</f>
-        <v>-47</v>
-      </c>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="27"/>
     </row>
     <row r="8" s="20" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="25"/>
@@ -79561,7 +79458,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G4:G7">
+  <conditionalFormatting sqref="G4:G4">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -79569,7 +79466,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J4:J7">
+  <conditionalFormatting sqref="J4:J4">
     <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>0</formula>
     </cfRule>
@@ -79577,7 +79474,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M4:M7">
+  <conditionalFormatting sqref="M4:M4">
     <cfRule type="cellIs" priority="6" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Reduce workbook XML validation overhead
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4689" uniqueCount="1756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4685" uniqueCount="1755">
   <si>
     <t>유류비 계산(혼유, 지역화폐 등)</t>
   </si>
@@ -5359,9 +5359,6 @@
   </si>
   <si>
     <t>현행화 일자: 2026-08-02</t>
-  </si>
-  <si>
-    <t>가격변동</t>
   </si>
 </sst>
 </file>
@@ -75216,44 +75213,19 @@
       </c>
     </row>
     <row r="4" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A4" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>398</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>399</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>1755</v>
-      </c>
-      <c r="E4" s="23">
-        <v>1814</v>
-      </c>
-      <c r="F4" s="23">
-        <v>1814</v>
-      </c>
-      <c r="G4" s="23">
-        <f>IF(OR(E4="",F4=""),"",F4-E4)</f>
-        <v>0</v>
-      </c>
+      <c r="A4" s="21"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
       <c r="H4" s="23"/>
       <c r="I4" s="23"/>
-      <c r="J4" s="23" t="str">
-        <f>IF(OR(H4="",I4=""),"",I4-H4)</f>
-        <v/>
-      </c>
-      <c r="K4" s="23">
-        <v>1793</v>
-      </c>
-      <c r="L4" s="23">
-        <v>1803</v>
-      </c>
-      <c r="M4" s="23">
-        <f>IF(OR(K4="",L4=""),"",L4-K4)</f>
-        <v>10</v>
-      </c>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
     </row>
     <row r="5" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
       <c r="A5" s="21"/>

</xml_diff>

<commit_message>
Validate retained workbook metadata
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4685" uniqueCount="1755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4737" uniqueCount="1756">
   <si>
     <t>유류비 계산(혼유, 지역화폐 등)</t>
   </si>
@@ -5359,6 +5359,9 @@
   </si>
   <si>
     <t>현행화 일자: 2026-08-02</t>
+  </si>
+  <si>
+    <t>가격변동</t>
   </si>
 </sst>
 </file>
@@ -13905,35 +13908,35 @@
         <v>92105</v>
       </c>
     </row>
-    <row r="103" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="103" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A103" s="12">
         <f t="shared" si="13"/>
         <v>89</v>
       </c>
       <c r="B103" s="12" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C103" s="12" t="s">
-        <v>197</v>
+        <v>235</v>
       </c>
       <c r="D103" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E103" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F103" s="12" t="s">
-        <v>198</v>
+        <v>236</v>
       </c>
       <c r="G103" s="13">
-        <v>1886</v>
+        <v>1824</v>
       </c>
       <c r="H103" s="13">
-        <v>2250</v>
+        <v>2328</v>
       </c>
       <c r="I103" s="13"/>
       <c r="J103" s="13">
-        <v>1876</v>
+        <v>1798</v>
       </c>
       <c r="K103" s="13">
         <f t="shared" si="14"/>
@@ -13941,23 +13944,23 @@
       </c>
       <c r="L103" s="13">
         <f t="shared" si="15"/>
-        <v>1886</v>
+        <v>1824</v>
       </c>
       <c r="M103" s="13">
         <f t="shared" si="16"/>
-        <v>2250</v>
+        <v>2328</v>
       </c>
       <c r="N103" s="13">
         <f t="shared" si="17"/>
-        <v>1876</v>
+        <v>1798</v>
       </c>
       <c r="O103" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 47,150원 / 고급유 45,000원</v>
+        <v>휘발유 45,600원 / 고급유 46,560원</v>
       </c>
       <c r="P103" s="13">
         <f t="shared" si="19"/>
-        <v>92150</v>
+        <v>92160</v>
       </c>
       <c r="Q103" s="13"/>
       <c r="R103" s="14">
@@ -13970,50 +13973,50 @@
       </c>
       <c r="T103" s="13">
         <f t="shared" si="22"/>
-        <v>92150</v>
+        <v>92160</v>
       </c>
       <c r="U103" s="13">
         <f t="shared" si="23"/>
-        <v>2047.7777777777778</v>
+        <v>2048</v>
       </c>
       <c r="V103" s="13">
         <f t="shared" si="24"/>
-        <v>2047.7777777777778</v>
+        <v>2048</v>
       </c>
       <c r="W103" s="15">
         <f t="shared" si="25"/>
-        <v>92150</v>
-      </c>
-    </row>
-    <row r="104" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+        <v>92160</v>
+      </c>
+    </row>
+    <row r="104" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A104" s="12">
         <f t="shared" si="13"/>
         <v>90</v>
       </c>
       <c r="B104" s="12" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C104" s="12" t="s">
-        <v>235</v>
+        <v>201</v>
       </c>
       <c r="D104" s="16" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E104" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F104" s="12" t="s">
-        <v>236</v>
+        <v>202</v>
       </c>
       <c r="G104" s="13">
-        <v>1824</v>
+        <v>1835</v>
       </c>
       <c r="H104" s="13">
-        <v>2328</v>
+        <v>2315</v>
       </c>
       <c r="I104" s="13"/>
       <c r="J104" s="13">
-        <v>1798</v>
+        <v>1799</v>
       </c>
       <c r="K104" s="13">
         <f t="shared" si="14"/>
@@ -14021,23 +14024,23 @@
       </c>
       <c r="L104" s="13">
         <f t="shared" si="15"/>
-        <v>1824</v>
+        <v>1835</v>
       </c>
       <c r="M104" s="13">
         <f t="shared" si="16"/>
-        <v>2328</v>
+        <v>2315</v>
       </c>
       <c r="N104" s="13">
         <f t="shared" si="17"/>
-        <v>1798</v>
+        <v>1799</v>
       </c>
       <c r="O104" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 45,600원 / 고급유 46,560원</v>
+        <v>휘발유 45,875원 / 고급유 46,300원</v>
       </c>
       <c r="P104" s="13">
         <f t="shared" si="19"/>
-        <v>92160</v>
+        <v>92175</v>
       </c>
       <c r="Q104" s="13"/>
       <c r="R104" s="14">
@@ -14050,31 +14053,31 @@
       </c>
       <c r="T104" s="13">
         <f t="shared" si="22"/>
-        <v>92160</v>
+        <v>92175</v>
       </c>
       <c r="U104" s="13">
         <f t="shared" si="23"/>
-        <v>2048</v>
+        <v>2048.3333333333335</v>
       </c>
       <c r="V104" s="13">
         <f t="shared" si="24"/>
-        <v>2048</v>
+        <v>2048.3333333333335</v>
       </c>
       <c r="W104" s="15">
         <f t="shared" si="25"/>
-        <v>92160</v>
+        <v>92175</v>
       </c>
     </row>
     <row r="105" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A105" s="12">
         <f t="shared" si="13"/>
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B105" s="12" t="s">
         <v>10</v>
       </c>
       <c r="C105" s="12" t="s">
-        <v>201</v>
+        <v>274</v>
       </c>
       <c r="D105" s="16" t="s">
         <v>71</v>
@@ -14083,7 +14086,7 @@
         <v>26</v>
       </c>
       <c r="F105" s="12" t="s">
-        <v>202</v>
+        <v>275</v>
       </c>
       <c r="G105" s="13">
         <v>1835</v>
@@ -14093,7 +14096,7 @@
       </c>
       <c r="I105" s="13"/>
       <c r="J105" s="13">
-        <v>1799</v>
+        <v>1815</v>
       </c>
       <c r="K105" s="13">
         <f t="shared" si="14"/>
@@ -14109,7 +14112,7 @@
       </c>
       <c r="N105" s="13">
         <f t="shared" si="17"/>
-        <v>1799</v>
+        <v>1815</v>
       </c>
       <c r="O105" s="13" t="str">
         <f t="shared" si="18"/>
@@ -14145,16 +14148,16 @@
         <v>92175</v>
       </c>
     </row>
-    <row r="106" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="106" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A106" s="12">
         <f t="shared" si="13"/>
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B106" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C106" s="12" t="s">
-        <v>274</v>
+        <v>205</v>
       </c>
       <c r="D106" s="16" t="s">
         <v>71</v>
@@ -14163,17 +14166,17 @@
         <v>26</v>
       </c>
       <c r="F106" s="12" t="s">
-        <v>275</v>
+        <v>206</v>
       </c>
       <c r="G106" s="13">
-        <v>1835</v>
+        <v>1845</v>
       </c>
       <c r="H106" s="13">
-        <v>2315</v>
+        <v>2303</v>
       </c>
       <c r="I106" s="13"/>
       <c r="J106" s="13">
-        <v>1815</v>
+        <v>1849</v>
       </c>
       <c r="K106" s="13">
         <f t="shared" si="14"/>
@@ -14181,23 +14184,23 @@
       </c>
       <c r="L106" s="13">
         <f t="shared" si="15"/>
-        <v>1835</v>
+        <v>1845</v>
       </c>
       <c r="M106" s="13">
         <f t="shared" si="16"/>
-        <v>2315</v>
+        <v>2303</v>
       </c>
       <c r="N106" s="13">
         <f t="shared" si="17"/>
-        <v>1815</v>
+        <v>1849</v>
       </c>
       <c r="O106" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 45,875원 / 고급유 46,300원</v>
+        <v>휘발유 46,125원 / 고급유 46,060원</v>
       </c>
       <c r="P106" s="13">
         <f t="shared" si="19"/>
-        <v>92175</v>
+        <v>92185</v>
       </c>
       <c r="Q106" s="13"/>
       <c r="R106" s="14">
@@ -14210,50 +14213,50 @@
       </c>
       <c r="T106" s="13">
         <f t="shared" si="22"/>
-        <v>92175</v>
+        <v>92185</v>
       </c>
       <c r="U106" s="13">
         <f t="shared" si="23"/>
-        <v>2048.3333333333335</v>
+        <v>2048.5555555555557</v>
       </c>
       <c r="V106" s="13">
         <f t="shared" si="24"/>
-        <v>2048.3333333333335</v>
+        <v>2048.5555555555557</v>
       </c>
       <c r="W106" s="15">
         <f t="shared" si="25"/>
-        <v>92175</v>
-      </c>
-    </row>
-    <row r="107" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+        <v>92185</v>
+      </c>
+    </row>
+    <row r="107" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A107" s="12">
         <f t="shared" si="13"/>
         <v>93</v>
       </c>
       <c r="B107" s="12" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C107" s="12" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="D107" s="16" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E107" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F107" s="12" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="G107" s="13">
-        <v>1845</v>
+        <v>1814</v>
       </c>
       <c r="H107" s="13">
-        <v>2303</v>
+        <v>2346</v>
       </c>
       <c r="I107" s="13"/>
       <c r="J107" s="13">
-        <v>1849</v>
+        <v>1808</v>
       </c>
       <c r="K107" s="13">
         <f t="shared" si="14"/>
@@ -14261,23 +14264,23 @@
       </c>
       <c r="L107" s="13">
         <f t="shared" si="15"/>
-        <v>1845</v>
+        <v>1814</v>
       </c>
       <c r="M107" s="13">
         <f t="shared" si="16"/>
-        <v>2303</v>
+        <v>2346</v>
       </c>
       <c r="N107" s="13">
         <f t="shared" si="17"/>
-        <v>1849</v>
+        <v>1808</v>
       </c>
       <c r="O107" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 46,125원 / 고급유 46,060원</v>
+        <v>휘발유 45,350원 / 고급유 46,920원</v>
       </c>
       <c r="P107" s="13">
         <f t="shared" si="19"/>
-        <v>92185</v>
+        <v>92270</v>
       </c>
       <c r="Q107" s="13"/>
       <c r="R107" s="14">
@@ -14290,22 +14293,22 @@
       </c>
       <c r="T107" s="13">
         <f t="shared" si="22"/>
-        <v>92185</v>
+        <v>92270</v>
       </c>
       <c r="U107" s="13">
         <f t="shared" si="23"/>
-        <v>2048.5555555555557</v>
+        <v>2050.4444444444443</v>
       </c>
       <c r="V107" s="13">
         <f t="shared" si="24"/>
-        <v>2048.5555555555557</v>
+        <v>2050.4444444444443</v>
       </c>
       <c r="W107" s="15">
         <f t="shared" si="25"/>
-        <v>92185</v>
-      </c>
-    </row>
-    <row r="108" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+        <v>92270</v>
+      </c>
+    </row>
+    <row r="108" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A108" s="12">
         <f t="shared" si="13"/>
         <v>94</v>
@@ -14314,26 +14317,26 @@
         <v>6</v>
       </c>
       <c r="C108" s="12" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D108" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E108" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F108" s="12" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G108" s="13">
-        <v>1814</v>
+        <v>1815</v>
       </c>
       <c r="H108" s="13">
-        <v>2346</v>
+        <v>2345</v>
       </c>
       <c r="I108" s="13"/>
       <c r="J108" s="13">
-        <v>1808</v>
+        <v>1799</v>
       </c>
       <c r="K108" s="13">
         <f t="shared" si="14"/>
@@ -14341,23 +14344,23 @@
       </c>
       <c r="L108" s="13">
         <f t="shared" si="15"/>
-        <v>1814</v>
+        <v>1815</v>
       </c>
       <c r="M108" s="13">
         <f t="shared" si="16"/>
-        <v>2346</v>
+        <v>2345</v>
       </c>
       <c r="N108" s="13">
         <f t="shared" si="17"/>
-        <v>1808</v>
+        <v>1799</v>
       </c>
       <c r="O108" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 45,350원 / 고급유 46,920원</v>
+        <v>휘발유 45,375원 / 고급유 46,900원</v>
       </c>
       <c r="P108" s="13">
         <f t="shared" si="19"/>
-        <v>92270</v>
+        <v>92275</v>
       </c>
       <c r="Q108" s="13"/>
       <c r="R108" s="14">
@@ -14370,19 +14373,19 @@
       </c>
       <c r="T108" s="13">
         <f t="shared" si="22"/>
-        <v>92270</v>
+        <v>92275</v>
       </c>
       <c r="U108" s="13">
         <f t="shared" si="23"/>
-        <v>2050.4444444444443</v>
+        <v>2050.5555555555557</v>
       </c>
       <c r="V108" s="13">
         <f t="shared" si="24"/>
-        <v>2050.4444444444443</v>
+        <v>2050.5555555555557</v>
       </c>
       <c r="W108" s="15">
         <f t="shared" si="25"/>
-        <v>92270</v>
+        <v>92275</v>
       </c>
     </row>
     <row r="109" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
@@ -14391,53 +14394,53 @@
         <v>95</v>
       </c>
       <c r="B109" s="12" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C109" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D109" s="16" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E109" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F109" s="12" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G109" s="13">
-        <v>1815</v>
+        <v>1854</v>
       </c>
       <c r="H109" s="13">
-        <v>2345</v>
+        <v>2319</v>
       </c>
       <c r="I109" s="13"/>
       <c r="J109" s="13">
-        <v>1799</v>
+        <v>1842</v>
       </c>
       <c r="K109" s="13">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="L109" s="13">
         <f t="shared" si="15"/>
-        <v>1815</v>
+        <v>1844</v>
       </c>
       <c r="M109" s="13">
         <f t="shared" si="16"/>
-        <v>2345</v>
+        <v>2309</v>
       </c>
       <c r="N109" s="13">
         <f t="shared" si="17"/>
-        <v>1799</v>
+        <v>1832</v>
       </c>
       <c r="O109" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 45,375원 / 고급유 46,900원</v>
+        <v>휘발유 46,100원 / 고급유 46,180원</v>
       </c>
       <c r="P109" s="13">
         <f t="shared" si="19"/>
-        <v>92275</v>
+        <v>92280</v>
       </c>
       <c r="Q109" s="13"/>
       <c r="R109" s="14">
@@ -14450,31 +14453,31 @@
       </c>
       <c r="T109" s="13">
         <f t="shared" si="22"/>
-        <v>92275</v>
+        <v>92280</v>
       </c>
       <c r="U109" s="13">
         <f t="shared" si="23"/>
-        <v>2050.5555555555557</v>
+        <v>2050.6666666666665</v>
       </c>
       <c r="V109" s="13">
         <f t="shared" si="24"/>
-        <v>2050.5555555555557</v>
+        <v>2050.6666666666665</v>
       </c>
       <c r="W109" s="15">
         <f t="shared" si="25"/>
-        <v>92275</v>
+        <v>92280</v>
       </c>
     </row>
     <row r="110" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A110" s="12">
         <f t="shared" si="13"/>
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B110" s="12" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C110" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D110" s="16" t="s">
         <v>52</v>
@@ -14483,7 +14486,7 @@
         <v>26</v>
       </c>
       <c r="F110" s="12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G110" s="13">
         <v>1854</v>
@@ -14493,7 +14496,7 @@
       </c>
       <c r="I110" s="13"/>
       <c r="J110" s="13">
-        <v>1842</v>
+        <v>1844</v>
       </c>
       <c r="K110" s="13">
         <f t="shared" si="14"/>
@@ -14509,7 +14512,7 @@
       </c>
       <c r="N110" s="13">
         <f t="shared" si="17"/>
-        <v>1832</v>
+        <v>1834</v>
       </c>
       <c r="O110" s="13" t="str">
         <f t="shared" si="18"/>
@@ -14545,59 +14548,59 @@
         <v>92280</v>
       </c>
     </row>
-    <row r="111" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="111" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A111" s="12">
         <f t="shared" si="13"/>
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B111" s="12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C111" s="12" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D111" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E111" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F111" s="12" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="G111" s="13">
         <v>1854</v>
       </c>
       <c r="H111" s="13">
-        <v>2319</v>
+        <v>2299</v>
       </c>
       <c r="I111" s="13"/>
       <c r="J111" s="13">
-        <v>1844</v>
+        <v>1842</v>
       </c>
       <c r="K111" s="13">
         <f t="shared" si="14"/>
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="L111" s="13">
         <f t="shared" si="15"/>
-        <v>1844</v>
+        <v>1854</v>
       </c>
       <c r="M111" s="13">
         <f t="shared" si="16"/>
-        <v>2309</v>
+        <v>2299</v>
       </c>
       <c r="N111" s="13">
         <f t="shared" si="17"/>
-        <v>1834</v>
+        <v>1842</v>
       </c>
       <c r="O111" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 46,100원 / 고급유 46,180원</v>
+        <v>휘발유 46,350원 / 고급유 45,980원</v>
       </c>
       <c r="P111" s="13">
         <f t="shared" si="19"/>
-        <v>92280</v>
+        <v>92330</v>
       </c>
       <c r="Q111" s="13"/>
       <c r="R111" s="14">
@@ -14610,50 +14613,50 @@
       </c>
       <c r="T111" s="13">
         <f t="shared" si="22"/>
-        <v>92280</v>
+        <v>92330</v>
       </c>
       <c r="U111" s="13">
         <f t="shared" si="23"/>
-        <v>2050.6666666666665</v>
+        <v>2051.7777777777778</v>
       </c>
       <c r="V111" s="13">
         <f t="shared" si="24"/>
-        <v>2050.6666666666665</v>
+        <v>2051.7777777777778</v>
       </c>
       <c r="W111" s="15">
         <f t="shared" si="25"/>
-        <v>92280</v>
-      </c>
-    </row>
-    <row r="112" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+        <v>92330</v>
+      </c>
+    </row>
+    <row r="112" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A112" s="12">
         <f t="shared" si="13"/>
         <v>98</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C112" s="12" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="D112" s="16" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E112" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F112" s="12" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="G112" s="13">
-        <v>1854</v>
+        <v>1833</v>
       </c>
       <c r="H112" s="13">
-        <v>2299</v>
+        <v>2328</v>
       </c>
       <c r="I112" s="13"/>
       <c r="J112" s="13">
-        <v>1842</v>
+        <v>1819</v>
       </c>
       <c r="K112" s="13">
         <f t="shared" si="14"/>
@@ -14661,23 +14664,23 @@
       </c>
       <c r="L112" s="13">
         <f t="shared" si="15"/>
-        <v>1854</v>
+        <v>1833</v>
       </c>
       <c r="M112" s="13">
         <f t="shared" si="16"/>
-        <v>2299</v>
+        <v>2328</v>
       </c>
       <c r="N112" s="13">
         <f t="shared" si="17"/>
-        <v>1842</v>
+        <v>1819</v>
       </c>
       <c r="O112" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 46,350원 / 고급유 45,980원</v>
+        <v>휘발유 45,825원 / 고급유 46,560원</v>
       </c>
       <c r="P112" s="13">
         <f t="shared" si="19"/>
-        <v>92330</v>
+        <v>92385</v>
       </c>
       <c r="Q112" s="13"/>
       <c r="R112" s="14">
@@ -14690,22 +14693,22 @@
       </c>
       <c r="T112" s="13">
         <f t="shared" si="22"/>
-        <v>92330</v>
+        <v>92385</v>
       </c>
       <c r="U112" s="13">
         <f t="shared" si="23"/>
-        <v>2051.7777777777778</v>
+        <v>2053</v>
       </c>
       <c r="V112" s="13">
         <f t="shared" si="24"/>
-        <v>2051.7777777777778</v>
+        <v>2053</v>
       </c>
       <c r="W112" s="15">
         <f t="shared" si="25"/>
-        <v>92330</v>
-      </c>
-    </row>
-    <row r="113" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+        <v>92385</v>
+      </c>
+    </row>
+    <row r="113" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A113" s="12">
         <f t="shared" si="13"/>
         <v>99</v>
@@ -14714,50 +14717,52 @@
         <v>6</v>
       </c>
       <c r="C113" s="12" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D113" s="16" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E113" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F113" s="12" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G113" s="13">
-        <v>1833</v>
+        <v>1848</v>
       </c>
       <c r="H113" s="13">
-        <v>2328</v>
-      </c>
-      <c r="I113" s="13"/>
+        <v>2332</v>
+      </c>
+      <c r="I113" s="13" t="s">
+        <v>47</v>
+      </c>
       <c r="J113" s="13">
-        <v>1819</v>
+        <v>1838</v>
       </c>
       <c r="K113" s="13">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="L113" s="13">
         <f t="shared" si="15"/>
-        <v>1833</v>
+        <v>1838</v>
       </c>
       <c r="M113" s="13">
         <f t="shared" si="16"/>
-        <v>2328</v>
+        <v>2322</v>
       </c>
       <c r="N113" s="13">
         <f t="shared" si="17"/>
-        <v>1819</v>
+        <v>1828</v>
       </c>
       <c r="O113" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 45,825원 / 고급유 46,560원</v>
+        <v>휘발유 45,950원 / 고급유 46,440원</v>
       </c>
       <c r="P113" s="13">
         <f t="shared" si="19"/>
-        <v>92385</v>
+        <v>92390</v>
       </c>
       <c r="Q113" s="13"/>
       <c r="R113" s="14">
@@ -14770,31 +14775,31 @@
       </c>
       <c r="T113" s="13">
         <f t="shared" si="22"/>
-        <v>92385</v>
+        <v>92390</v>
       </c>
       <c r="U113" s="13">
         <f t="shared" si="23"/>
-        <v>2053</v>
+        <v>2053.1111111111113</v>
       </c>
       <c r="V113" s="13">
         <f t="shared" si="24"/>
-        <v>2053</v>
+        <v>2053.1111111111113</v>
       </c>
       <c r="W113" s="15">
         <f t="shared" si="25"/>
-        <v>92385</v>
-      </c>
-    </row>
-    <row r="114" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+        <v>92390</v>
+      </c>
+    </row>
+    <row r="114" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A114" s="12">
         <f t="shared" si="13"/>
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B114" s="12" t="s">
         <v>6</v>
       </c>
       <c r="C114" s="12" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D114" s="16" t="s">
         <v>52</v>
@@ -14803,7 +14808,7 @@
         <v>26</v>
       </c>
       <c r="F114" s="12" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="G114" s="13">
         <v>1848</v>
@@ -14867,16 +14872,16 @@
         <v>92390</v>
       </c>
     </row>
-    <row r="115" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="115" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A115" s="12">
         <f t="shared" si="13"/>
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B115" s="12" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C115" s="12" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="D115" s="16" t="s">
         <v>52</v>
@@ -14885,43 +14890,41 @@
         <v>26</v>
       </c>
       <c r="F115" s="12" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="G115" s="13">
-        <v>1848</v>
+        <v>1896</v>
       </c>
       <c r="H115" s="13">
-        <v>2332</v>
-      </c>
-      <c r="I115" s="13" t="s">
-        <v>47</v>
-      </c>
+        <v>2250</v>
+      </c>
+      <c r="I115" s="13"/>
       <c r="J115" s="13">
-        <v>1838</v>
+        <v>1876</v>
       </c>
       <c r="K115" s="13">
         <f t="shared" si="14"/>
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="L115" s="13">
         <f t="shared" si="15"/>
-        <v>1838</v>
+        <v>1896</v>
       </c>
       <c r="M115" s="13">
         <f t="shared" si="16"/>
-        <v>2322</v>
+        <v>2250</v>
       </c>
       <c r="N115" s="13">
         <f t="shared" si="17"/>
-        <v>1828</v>
+        <v>1876</v>
       </c>
       <c r="O115" s="13" t="str">
         <f t="shared" si="18"/>
-        <v>휘발유 45,950원 / 고급유 46,440원</v>
+        <v>휘발유 47,400원 / 고급유 45,000원</v>
       </c>
       <c r="P115" s="13">
         <f t="shared" si="19"/>
-        <v>92390</v>
+        <v>92400</v>
       </c>
       <c r="Q115" s="13"/>
       <c r="R115" s="14">
@@ -14934,19 +14937,19 @@
       </c>
       <c r="T115" s="13">
         <f t="shared" si="22"/>
-        <v>92390</v>
+        <v>92400</v>
       </c>
       <c r="U115" s="13">
         <f t="shared" si="23"/>
-        <v>2053.1111111111113</v>
+        <v>2053.3333333333335</v>
       </c>
       <c r="V115" s="13">
         <f t="shared" si="24"/>
-        <v>2053.1111111111113</v>
+        <v>2053.3333333333335</v>
       </c>
       <c r="W115" s="15">
         <f t="shared" si="25"/>
-        <v>92390</v>
+        <v>92400</v>
       </c>
     </row>
     <row r="116" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
@@ -21517,7 +21520,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="198" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="198" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A198" s="12" t="str">
         <f t="shared" si="26"/>
         <v/>
@@ -21526,16 +21529,16 @@
         <v>18</v>
       </c>
       <c r="C198" s="12" t="s">
-        <v>470</v>
-      </c>
-      <c r="D198" s="12" t="s">
-        <v>49</v>
+        <v>408</v>
+      </c>
+      <c r="D198" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="E198" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F198" s="12" t="s">
-        <v>471</v>
+        <v>409</v>
       </c>
       <c r="G198" s="13">
         <v>1859</v>
@@ -21597,7 +21600,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="199" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="199" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A199" s="12" t="str">
         <f t="shared" si="26"/>
         <v/>
@@ -21606,16 +21609,16 @@
         <v>18</v>
       </c>
       <c r="C199" s="12" t="s">
-        <v>408</v>
-      </c>
-      <c r="D199" s="16" t="s">
-        <v>71</v>
+        <v>470</v>
+      </c>
+      <c r="D199" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E199" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F199" s="12" t="s">
-        <v>409</v>
+        <v>471</v>
       </c>
       <c r="G199" s="13">
         <v>1859</v>
@@ -21623,7 +21626,7 @@
       <c r="H199" s="13"/>
       <c r="I199" s="13"/>
       <c r="J199" s="13">
-        <v>1849</v>
+        <v>1869</v>
       </c>
       <c r="K199" s="13">
         <f t="shared" si="27"/>
@@ -21639,7 +21642,7 @@
       </c>
       <c r="N199" s="13">
         <f t="shared" si="30"/>
-        <v>1849</v>
+        <v>1869</v>
       </c>
       <c r="O199" s="13" t="str">
         <f t="shared" si="31"/>
@@ -23143,7 +23146,7 @@
       <c r="H218" s="13"/>
       <c r="I218" s="13"/>
       <c r="J218" s="13">
-        <v>1849</v>
+        <v>1854</v>
       </c>
       <c r="K218" s="13">
         <f t="shared" si="40"/>
@@ -23159,7 +23162,7 @@
       </c>
       <c r="N218" s="13">
         <f t="shared" si="43"/>
-        <v>1849</v>
+        <v>1854</v>
       </c>
       <c r="O218" s="13" t="str">
         <f t="shared" si="44"/>
@@ -24797,7 +24800,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="239" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="239" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A239" s="12" t="str">
         <f t="shared" si="39"/>
         <v/>
@@ -24806,16 +24809,16 @@
         <v>16</v>
       </c>
       <c r="C239" s="12" t="s">
-        <v>474</v>
+        <v>597</v>
       </c>
       <c r="D239" s="16" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E239" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F239" s="12" t="s">
-        <v>475</v>
+        <v>598</v>
       </c>
       <c r="G239" s="13">
         <v>1880</v>
@@ -24823,7 +24826,7 @@
       <c r="H239" s="13"/>
       <c r="I239" s="13"/>
       <c r="J239" s="13">
-        <v>1860</v>
+        <v>1880</v>
       </c>
       <c r="K239" s="13">
         <f t="shared" si="40"/>
@@ -24839,7 +24842,7 @@
       </c>
       <c r="N239" s="13">
         <f t="shared" si="43"/>
-        <v>1860</v>
+        <v>1880</v>
       </c>
       <c r="O239" s="13" t="str">
         <f t="shared" si="44"/>
@@ -24877,7 +24880,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="240" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="240" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A240" s="12" t="str">
         <f t="shared" si="39"/>
         <v/>
@@ -24886,16 +24889,16 @@
         <v>16</v>
       </c>
       <c r="C240" s="12" t="s">
-        <v>597</v>
+        <v>474</v>
       </c>
       <c r="D240" s="16" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E240" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F240" s="12" t="s">
-        <v>598</v>
+        <v>475</v>
       </c>
       <c r="G240" s="13">
         <v>1880</v>
@@ -24903,7 +24906,7 @@
       <c r="H240" s="13"/>
       <c r="I240" s="13"/>
       <c r="J240" s="13">
-        <v>1880</v>
+        <v>1890</v>
       </c>
       <c r="K240" s="13">
         <f t="shared" si="40"/>
@@ -24919,7 +24922,7 @@
       </c>
       <c r="N240" s="13">
         <f t="shared" si="43"/>
-        <v>1880</v>
+        <v>1890</v>
       </c>
       <c r="O240" s="13" t="str">
         <f t="shared" si="44"/>
@@ -26743,7 +26746,7 @@
       <c r="H263" s="13"/>
       <c r="I263" s="13"/>
       <c r="J263" s="13">
-        <v>1847</v>
+        <v>1867</v>
       </c>
       <c r="K263" s="13">
         <f t="shared" si="40"/>
@@ -26759,7 +26762,7 @@
       </c>
       <c r="N263" s="13">
         <f t="shared" si="43"/>
-        <v>1847</v>
+        <v>1867</v>
       </c>
       <c r="O263" s="13" t="str">
         <f t="shared" si="44"/>
@@ -27043,27 +27046,27 @@
         <v/>
       </c>
       <c r="B267" s="12" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C267" s="12" t="s">
-        <v>531</v>
+        <v>599</v>
       </c>
       <c r="D267" s="16" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E267" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F267" s="12" t="s">
-        <v>532</v>
+        <v>600</v>
       </c>
       <c r="G267" s="13">
-        <v>1890</v>
+        <v>1848</v>
       </c>
       <c r="H267" s="13"/>
       <c r="I267" s="13"/>
       <c r="J267" s="13">
-        <v>1880</v>
+        <v>1838</v>
       </c>
       <c r="K267" s="13">
         <f t="shared" si="40"/>
@@ -27071,7 +27074,7 @@
       </c>
       <c r="L267" s="13">
         <f t="shared" si="41"/>
-        <v>1890</v>
+        <v>1848</v>
       </c>
       <c r="M267" s="13" t="str">
         <f t="shared" si="42"/>
@@ -27079,7 +27082,7 @@
       </c>
       <c r="N267" s="13">
         <f t="shared" si="43"/>
-        <v>1880</v>
+        <v>1838</v>
       </c>
       <c r="O267" s="13" t="str">
         <f t="shared" si="44"/>
@@ -27117,7 +27120,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="268" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="268" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A268" s="12" t="str">
         <f t="shared" si="39"/>
         <v/>
@@ -27126,16 +27129,16 @@
         <v>18</v>
       </c>
       <c r="C268" s="12" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D268" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E268" s="12" t="s">
         <v>62</v>
       </c>
       <c r="F268" s="12" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="G268" s="13">
         <v>1890</v>
@@ -27197,7 +27200,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="269" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="269" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A269" s="12" t="str">
         <f t="shared" si="39"/>
         <v/>
@@ -27206,16 +27209,16 @@
         <v>18</v>
       </c>
       <c r="C269" s="12" t="s">
-        <v>535</v>
-      </c>
-      <c r="D269" s="12" t="s">
-        <v>49</v>
+        <v>533</v>
+      </c>
+      <c r="D269" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E269" s="12" t="s">
         <v>62</v>
       </c>
       <c r="F269" s="12" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="G269" s="13">
         <v>1890</v>
@@ -27223,7 +27226,7 @@
       <c r="H269" s="13"/>
       <c r="I269" s="13"/>
       <c r="J269" s="13">
-        <v>1890</v>
+        <v>1880</v>
       </c>
       <c r="K269" s="13">
         <f t="shared" si="40"/>
@@ -27239,7 +27242,7 @@
       </c>
       <c r="N269" s="13">
         <f t="shared" si="43"/>
-        <v>1890</v>
+        <v>1880</v>
       </c>
       <c r="O269" s="13" t="str">
         <f t="shared" si="44"/>
@@ -27277,25 +27280,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="270" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="270" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A270" s="12" t="str">
         <f t="shared" si="39"/>
         <v/>
       </c>
       <c r="B270" s="12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C270" s="12" t="s">
-        <v>658</v>
-      </c>
-      <c r="D270" s="16" t="s">
-        <v>52</v>
+        <v>535</v>
+      </c>
+      <c r="D270" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E270" s="12" t="s">
         <v>62</v>
       </c>
       <c r="F270" s="12" t="s">
-        <v>659</v>
+        <v>536</v>
       </c>
       <c r="G270" s="13">
         <v>1890</v>
@@ -27366,16 +27369,16 @@
         <v>16</v>
       </c>
       <c r="C271" s="12" t="s">
-        <v>595</v>
+        <v>658</v>
       </c>
       <c r="D271" s="16" t="s">
         <v>52</v>
       </c>
       <c r="E271" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F271" s="12" t="s">
-        <v>596</v>
+        <v>659</v>
       </c>
       <c r="G271" s="13">
         <v>1890</v>
@@ -27383,7 +27386,7 @@
       <c r="H271" s="13"/>
       <c r="I271" s="13"/>
       <c r="J271" s="13">
-        <v>1900</v>
+        <v>1890</v>
       </c>
       <c r="K271" s="13">
         <f t="shared" ref="K271:K334" si="53">IF(AND(IFERROR(SEARCH("현대오일뱅크",$C271),0)&gt;0,IFERROR(SEARCH("직영",$C271),0)&gt;0),$B$13,0)</f>
@@ -27399,7 +27402,7 @@
       </c>
       <c r="N271" s="13">
         <f t="shared" ref="N271:N334" si="56">IF($J271="","",$J271+$K271)</f>
-        <v>1900</v>
+        <v>1890</v>
       </c>
       <c r="O271" s="13" t="str">
         <f t="shared" ref="O271:O334" si="57">IF($B$10=0,"",IFERROR(IF($B$4&gt;0,"휘발유 "&amp;TEXT(IF($L271="",1/0,$L271*$B$4),"#,##0")&amp;"원","")&amp;IF($B$5&gt;0,IF($B$4&gt;0," / ","")&amp;"고급유 "&amp;TEXT(IF($M271="",1/0,$M271*$B$5),"#,##0")&amp;"원","")&amp;IF($B$6&gt;0,IF(OR($B$4&gt;0,$B$5&gt;0)," / ","")&amp;"경유 "&amp;TEXT(IF($N271="",1/0,$N271*$B$6),"#,##0")&amp;"원",""),""))</f>
@@ -27443,27 +27446,27 @@
         <v/>
       </c>
       <c r="B272" s="12" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C272" s="12" t="s">
-        <v>622</v>
-      </c>
-      <c r="D272" s="12" t="s">
-        <v>49</v>
+        <v>595</v>
+      </c>
+      <c r="D272" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E272" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F272" s="12" t="s">
-        <v>623</v>
+        <v>596</v>
       </c>
       <c r="G272" s="13">
-        <v>1849</v>
+        <v>1890</v>
       </c>
       <c r="H272" s="13"/>
       <c r="I272" s="13"/>
       <c r="J272" s="13">
-        <v>1799</v>
+        <v>1900</v>
       </c>
       <c r="K272" s="13">
         <f t="shared" si="53"/>
@@ -27471,7 +27474,7 @@
       </c>
       <c r="L272" s="13">
         <f t="shared" si="54"/>
-        <v>1849</v>
+        <v>1890</v>
       </c>
       <c r="M272" s="13" t="str">
         <f t="shared" si="55"/>
@@ -27479,7 +27482,7 @@
       </c>
       <c r="N272" s="13">
         <f t="shared" si="56"/>
-        <v>1799</v>
+        <v>1900</v>
       </c>
       <c r="O272" s="13" t="str">
         <f t="shared" si="57"/>
@@ -27517,25 +27520,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="273" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="273" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A273" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B273" s="12" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C273" s="12" t="s">
-        <v>539</v>
-      </c>
-      <c r="D273" s="16" t="s">
-        <v>52</v>
+        <v>622</v>
+      </c>
+      <c r="D273" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E273" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F273" s="12" t="s">
-        <v>540</v>
+        <v>623</v>
       </c>
       <c r="G273" s="13">
         <v>1849</v>
@@ -27603,19 +27606,19 @@
         <v/>
       </c>
       <c r="B274" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C274" s="12" t="s">
-        <v>553</v>
+        <v>539</v>
       </c>
       <c r="D274" s="16" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E274" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F274" s="12" t="s">
-        <v>554</v>
+        <v>540</v>
       </c>
       <c r="G274" s="13">
         <v>1849</v>
@@ -27623,7 +27626,7 @@
       <c r="H274" s="13"/>
       <c r="I274" s="13"/>
       <c r="J274" s="13">
-        <v>1809</v>
+        <v>1799</v>
       </c>
       <c r="K274" s="13">
         <f t="shared" si="53"/>
@@ -27639,7 +27642,7 @@
       </c>
       <c r="N274" s="13">
         <f t="shared" si="56"/>
-        <v>1809</v>
+        <v>1799</v>
       </c>
       <c r="O274" s="13" t="str">
         <f t="shared" si="57"/>
@@ -27677,7 +27680,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="275" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="275" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A275" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
@@ -27686,16 +27689,16 @@
         <v>10</v>
       </c>
       <c r="C275" s="12" t="s">
-        <v>616</v>
-      </c>
-      <c r="D275" s="12" t="s">
-        <v>49</v>
+        <v>553</v>
+      </c>
+      <c r="D275" s="16" t="s">
+        <v>59</v>
       </c>
       <c r="E275" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F275" s="12" t="s">
-        <v>617</v>
+        <v>554</v>
       </c>
       <c r="G275" s="13">
         <v>1849</v>
@@ -27703,7 +27706,7 @@
       <c r="H275" s="13"/>
       <c r="I275" s="13"/>
       <c r="J275" s="13">
-        <v>1819</v>
+        <v>1809</v>
       </c>
       <c r="K275" s="13">
         <f t="shared" si="53"/>
@@ -27719,7 +27722,7 @@
       </c>
       <c r="N275" s="13">
         <f t="shared" si="56"/>
-        <v>1819</v>
+        <v>1809</v>
       </c>
       <c r="O275" s="13" t="str">
         <f t="shared" si="57"/>
@@ -27757,25 +27760,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="276" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="276" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A276" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B276" s="12" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C276" s="12" t="s">
-        <v>545</v>
-      </c>
-      <c r="D276" s="16" t="s">
-        <v>59</v>
+        <v>616</v>
+      </c>
+      <c r="D276" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E276" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F276" s="12" t="s">
-        <v>546</v>
+        <v>617</v>
       </c>
       <c r="G276" s="13">
         <v>1849</v>
@@ -27783,7 +27786,7 @@
       <c r="H276" s="13"/>
       <c r="I276" s="13"/>
       <c r="J276" s="13">
-        <v>1834</v>
+        <v>1819</v>
       </c>
       <c r="K276" s="13">
         <f t="shared" si="53"/>
@@ -27799,7 +27802,7 @@
       </c>
       <c r="N276" s="13">
         <f t="shared" si="56"/>
-        <v>1834</v>
+        <v>1819</v>
       </c>
       <c r="O276" s="13" t="str">
         <f t="shared" si="57"/>
@@ -27837,7 +27840,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="277" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="277" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A277" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
@@ -27846,16 +27849,16 @@
         <v>6</v>
       </c>
       <c r="C277" s="12" t="s">
-        <v>547</v>
-      </c>
-      <c r="D277" s="12" t="s">
-        <v>49</v>
+        <v>545</v>
+      </c>
+      <c r="D277" s="16" t="s">
+        <v>59</v>
       </c>
       <c r="E277" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F277" s="12" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="G277" s="13">
         <v>1849</v>
@@ -27863,7 +27866,7 @@
       <c r="H277" s="13"/>
       <c r="I277" s="13"/>
       <c r="J277" s="13">
-        <v>1836</v>
+        <v>1834</v>
       </c>
       <c r="K277" s="13">
         <f t="shared" si="53"/>
@@ -27879,7 +27882,7 @@
       </c>
       <c r="N277" s="13">
         <f t="shared" si="56"/>
-        <v>1836</v>
+        <v>1834</v>
       </c>
       <c r="O277" s="13" t="str">
         <f t="shared" si="57"/>
@@ -27926,16 +27929,16 @@
         <v>6</v>
       </c>
       <c r="C278" s="12" t="s">
-        <v>549</v>
-      </c>
-      <c r="D278" s="16" t="s">
-        <v>52</v>
+        <v>547</v>
+      </c>
+      <c r="D278" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E278" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F278" s="12" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="G278" s="13">
         <v>1849</v>
@@ -27943,7 +27946,7 @@
       <c r="H278" s="13"/>
       <c r="I278" s="13"/>
       <c r="J278" s="13">
-        <v>1839</v>
+        <v>1836</v>
       </c>
       <c r="K278" s="13">
         <f t="shared" si="53"/>
@@ -27959,7 +27962,7 @@
       </c>
       <c r="N278" s="13">
         <f t="shared" si="56"/>
-        <v>1839</v>
+        <v>1836</v>
       </c>
       <c r="O278" s="13" t="str">
         <f t="shared" si="57"/>
@@ -27997,25 +28000,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="279" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="279" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A279" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B279" s="12" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C279" s="12" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="D279" s="16" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E279" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F279" s="12" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="G279" s="13">
         <v>1849</v>
@@ -28077,25 +28080,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="280" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="280" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A280" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B280" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C280" s="12" t="s">
-        <v>583</v>
+        <v>551</v>
       </c>
       <c r="D280" s="16" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E280" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F280" s="12" t="s">
-        <v>584</v>
+        <v>552</v>
       </c>
       <c r="G280" s="13">
         <v>1849</v>
@@ -28103,7 +28106,7 @@
       <c r="H280" s="13"/>
       <c r="I280" s="13"/>
       <c r="J280" s="13">
-        <v>1849</v>
+        <v>1839</v>
       </c>
       <c r="K280" s="13">
         <f t="shared" si="53"/>
@@ -28119,7 +28122,7 @@
       </c>
       <c r="N280" s="13">
         <f t="shared" si="56"/>
-        <v>1849</v>
+        <v>1839</v>
       </c>
       <c r="O280" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28157,7 +28160,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="281" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="281" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A281" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
@@ -28166,16 +28169,16 @@
         <v>10</v>
       </c>
       <c r="C281" s="12" t="s">
-        <v>644</v>
-      </c>
-      <c r="D281" s="12" t="s">
-        <v>45</v>
+        <v>583</v>
+      </c>
+      <c r="D281" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="E281" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F281" s="12" t="s">
-        <v>645</v>
+        <v>584</v>
       </c>
       <c r="G281" s="13">
         <v>1849</v>
@@ -28243,27 +28246,27 @@
         <v/>
       </c>
       <c r="B282" s="12" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C282" s="12" t="s">
-        <v>450</v>
-      </c>
-      <c r="D282" s="16" t="s">
-        <v>52</v>
+        <v>644</v>
+      </c>
+      <c r="D282" s="12" t="s">
+        <v>45</v>
       </c>
       <c r="E282" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F282" s="12" t="s">
-        <v>451</v>
+        <v>645</v>
       </c>
       <c r="G282" s="13">
-        <v>1892</v>
+        <v>1849</v>
       </c>
       <c r="H282" s="13"/>
       <c r="I282" s="13"/>
       <c r="J282" s="13">
-        <v>1882</v>
+        <v>1849</v>
       </c>
       <c r="K282" s="13">
         <f t="shared" si="53"/>
@@ -28271,7 +28274,7 @@
       </c>
       <c r="L282" s="13">
         <f t="shared" si="54"/>
-        <v>1892</v>
+        <v>1849</v>
       </c>
       <c r="M282" s="13" t="str">
         <f t="shared" si="55"/>
@@ -28279,7 +28282,7 @@
       </c>
       <c r="N282" s="13">
         <f t="shared" si="56"/>
-        <v>1882</v>
+        <v>1849</v>
       </c>
       <c r="O282" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28323,27 +28326,27 @@
         <v/>
       </c>
       <c r="B283" s="12" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C283" s="12" t="s">
-        <v>555</v>
-      </c>
-      <c r="D283" s="12" t="s">
-        <v>45</v>
+        <v>450</v>
+      </c>
+      <c r="D283" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E283" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F283" s="12" t="s">
-        <v>556</v>
+        <v>451</v>
       </c>
       <c r="G283" s="13">
-        <v>1852</v>
+        <v>1892</v>
       </c>
       <c r="H283" s="13"/>
       <c r="I283" s="13"/>
       <c r="J283" s="13">
-        <v>1839</v>
+        <v>1882</v>
       </c>
       <c r="K283" s="13">
         <f t="shared" si="53"/>
@@ -28351,7 +28354,7 @@
       </c>
       <c r="L283" s="13">
         <f t="shared" si="54"/>
-        <v>1852</v>
+        <v>1892</v>
       </c>
       <c r="M283" s="13" t="str">
         <f t="shared" si="55"/>
@@ -28359,7 +28362,7 @@
       </c>
       <c r="N283" s="13">
         <f t="shared" si="56"/>
-        <v>1839</v>
+        <v>1882</v>
       </c>
       <c r="O283" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28397,33 +28400,33 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="284" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="284" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A284" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B284" s="12" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C284" s="12" t="s">
-        <v>557</v>
-      </c>
-      <c r="D284" s="16" t="s">
-        <v>59</v>
+        <v>555</v>
+      </c>
+      <c r="D284" s="12" t="s">
+        <v>45</v>
       </c>
       <c r="E284" s="12" t="s">
         <v>62</v>
       </c>
       <c r="F284" s="12" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="G284" s="13">
-        <v>1895</v>
+        <v>1852</v>
       </c>
       <c r="H284" s="13"/>
       <c r="I284" s="13"/>
       <c r="J284" s="13">
-        <v>1850</v>
+        <v>1839</v>
       </c>
       <c r="K284" s="13">
         <f t="shared" si="53"/>
@@ -28431,7 +28434,7 @@
       </c>
       <c r="L284" s="13">
         <f t="shared" si="54"/>
-        <v>1895</v>
+        <v>1852</v>
       </c>
       <c r="M284" s="13" t="str">
         <f t="shared" si="55"/>
@@ -28439,7 +28442,7 @@
       </c>
       <c r="N284" s="13">
         <f t="shared" si="56"/>
-        <v>1850</v>
+        <v>1839</v>
       </c>
       <c r="O284" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28477,25 +28480,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="285" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="285" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A285" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B285" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C285" s="12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="D285" s="16" t="s">
         <v>59</v>
       </c>
       <c r="E285" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F285" s="12" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="G285" s="13">
         <v>1895</v>
@@ -28503,7 +28506,7 @@
       <c r="H285" s="13"/>
       <c r="I285" s="13"/>
       <c r="J285" s="13">
-        <v>1855</v>
+        <v>1850</v>
       </c>
       <c r="K285" s="13">
         <f t="shared" si="53"/>
@@ -28519,7 +28522,7 @@
       </c>
       <c r="N285" s="13">
         <f t="shared" si="56"/>
-        <v>1855</v>
+        <v>1850</v>
       </c>
       <c r="O285" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28566,16 +28569,16 @@
         <v>18</v>
       </c>
       <c r="C286" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="D286" s="16" t="s">
         <v>59</v>
       </c>
       <c r="E286" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F286" s="12" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="G286" s="13">
         <v>1895</v>
@@ -28583,7 +28586,7 @@
       <c r="H286" s="13"/>
       <c r="I286" s="13"/>
       <c r="J286" s="13">
-        <v>1875</v>
+        <v>1855</v>
       </c>
       <c r="K286" s="13">
         <f t="shared" si="53"/>
@@ -28599,7 +28602,7 @@
       </c>
       <c r="N286" s="13">
         <f t="shared" si="56"/>
-        <v>1875</v>
+        <v>1855</v>
       </c>
       <c r="O286" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28646,16 +28649,16 @@
         <v>18</v>
       </c>
       <c r="C287" s="12" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D287" s="16" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E287" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F287" s="12" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="G287" s="13">
         <v>1895</v>
@@ -28726,16 +28729,16 @@
         <v>18</v>
       </c>
       <c r="C288" s="12" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="D288" s="16" t="s">
         <v>71</v>
       </c>
       <c r="E288" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F288" s="12" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="G288" s="13">
         <v>1895</v>
@@ -28743,7 +28746,7 @@
       <c r="H288" s="13"/>
       <c r="I288" s="13"/>
       <c r="J288" s="13">
-        <v>1895</v>
+        <v>1875</v>
       </c>
       <c r="K288" s="13">
         <f t="shared" si="53"/>
@@ -28759,7 +28762,7 @@
       </c>
       <c r="N288" s="13">
         <f t="shared" si="56"/>
-        <v>1895</v>
+        <v>1875</v>
       </c>
       <c r="O288" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28803,27 +28806,27 @@
         <v/>
       </c>
       <c r="B289" s="12" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C289" s="12" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="D289" s="16" t="s">
         <v>71</v>
       </c>
       <c r="E289" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F289" s="12" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="G289" s="13">
-        <v>1854</v>
+        <v>1895</v>
       </c>
       <c r="H289" s="13"/>
       <c r="I289" s="13"/>
       <c r="J289" s="13">
-        <v>1818</v>
+        <v>1895</v>
       </c>
       <c r="K289" s="13">
         <f t="shared" si="53"/>
@@ -28831,7 +28834,7 @@
       </c>
       <c r="L289" s="13">
         <f t="shared" si="54"/>
-        <v>1854</v>
+        <v>1895</v>
       </c>
       <c r="M289" s="13" t="str">
         <f t="shared" si="55"/>
@@ -28839,7 +28842,7 @@
       </c>
       <c r="N289" s="13">
         <f t="shared" si="56"/>
-        <v>1818</v>
+        <v>1895</v>
       </c>
       <c r="O289" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28886,16 +28889,16 @@
         <v>10</v>
       </c>
       <c r="C290" s="12" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="D290" s="16" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E290" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F290" s="12" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="G290" s="13">
         <v>1854</v>
@@ -28903,7 +28906,7 @@
       <c r="H290" s="13"/>
       <c r="I290" s="13"/>
       <c r="J290" s="13">
-        <v>1837</v>
+        <v>1818</v>
       </c>
       <c r="K290" s="13">
         <f t="shared" si="53"/>
@@ -28919,7 +28922,7 @@
       </c>
       <c r="N290" s="13">
         <f t="shared" si="56"/>
-        <v>1837</v>
+        <v>1818</v>
       </c>
       <c r="O290" s="13" t="str">
         <f t="shared" si="57"/>
@@ -28963,27 +28966,27 @@
         <v/>
       </c>
       <c r="B291" s="12" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C291" s="12" t="s">
-        <v>577</v>
-      </c>
-      <c r="D291" s="12" t="s">
-        <v>49</v>
+        <v>571</v>
+      </c>
+      <c r="D291" s="16" t="s">
+        <v>59</v>
       </c>
       <c r="E291" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F291" s="12" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="G291" s="13">
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="H291" s="13"/>
       <c r="I291" s="13"/>
       <c r="J291" s="13">
-        <v>1825</v>
+        <v>1829</v>
       </c>
       <c r="K291" s="13">
         <f t="shared" si="53"/>
@@ -28991,7 +28994,7 @@
       </c>
       <c r="L291" s="13">
         <f t="shared" si="54"/>
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="M291" s="13" t="str">
         <f t="shared" si="55"/>
@@ -28999,7 +29002,7 @@
       </c>
       <c r="N291" s="13">
         <f t="shared" si="56"/>
-        <v>1825</v>
+        <v>1829</v>
       </c>
       <c r="O291" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29043,19 +29046,19 @@
         <v/>
       </c>
       <c r="B292" s="12" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C292" s="12" t="s">
-        <v>579</v>
-      </c>
-      <c r="D292" s="16" t="s">
-        <v>52</v>
+        <v>577</v>
+      </c>
+      <c r="D292" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E292" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F292" s="12" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="G292" s="13">
         <v>1855</v>
@@ -29063,7 +29066,7 @@
       <c r="H292" s="13"/>
       <c r="I292" s="13"/>
       <c r="J292" s="13">
-        <v>1839</v>
+        <v>1825</v>
       </c>
       <c r="K292" s="13">
         <f t="shared" si="53"/>
@@ -29079,7 +29082,7 @@
       </c>
       <c r="N292" s="13">
         <f t="shared" si="56"/>
-        <v>1839</v>
+        <v>1825</v>
       </c>
       <c r="O292" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29117,25 +29120,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="293" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="293" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A293" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B293" s="12" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C293" s="12" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="D293" s="16" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E293" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F293" s="12" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="G293" s="13">
         <v>1855</v>
@@ -29143,7 +29146,7 @@
       <c r="H293" s="13"/>
       <c r="I293" s="13"/>
       <c r="J293" s="13">
-        <v>1845</v>
+        <v>1839</v>
       </c>
       <c r="K293" s="13">
         <f t="shared" si="53"/>
@@ -29159,7 +29162,7 @@
       </c>
       <c r="N293" s="13">
         <f t="shared" si="56"/>
-        <v>1845</v>
+        <v>1839</v>
       </c>
       <c r="O293" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29197,33 +29200,33 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="294" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="294" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A294" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B294" s="12" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C294" s="12" t="s">
-        <v>585</v>
-      </c>
-      <c r="D294" s="12" t="s">
-        <v>49</v>
+        <v>581</v>
+      </c>
+      <c r="D294" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="E294" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F294" s="12" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="G294" s="13">
-        <v>1899</v>
+        <v>1855</v>
       </c>
       <c r="H294" s="13"/>
       <c r="I294" s="13"/>
       <c r="J294" s="13">
-        <v>1829</v>
+        <v>1845</v>
       </c>
       <c r="K294" s="13">
         <f t="shared" si="53"/>
@@ -29231,7 +29234,7 @@
       </c>
       <c r="L294" s="13">
         <f t="shared" si="54"/>
-        <v>1899</v>
+        <v>1855</v>
       </c>
       <c r="M294" s="13" t="str">
         <f t="shared" si="55"/>
@@ -29239,7 +29242,7 @@
       </c>
       <c r="N294" s="13">
         <f t="shared" si="56"/>
-        <v>1829</v>
+        <v>1845</v>
       </c>
       <c r="O294" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29286,16 +29289,16 @@
         <v>18</v>
       </c>
       <c r="C295" s="12" t="s">
-        <v>589</v>
-      </c>
-      <c r="D295" s="16" t="s">
-        <v>59</v>
+        <v>585</v>
+      </c>
+      <c r="D295" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E295" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F295" s="12" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="G295" s="13">
         <v>1899</v>
@@ -29303,7 +29306,7 @@
       <c r="H295" s="13"/>
       <c r="I295" s="13"/>
       <c r="J295" s="13">
-        <v>1869</v>
+        <v>1829</v>
       </c>
       <c r="K295" s="13">
         <f t="shared" si="53"/>
@@ -29319,7 +29322,7 @@
       </c>
       <c r="N295" s="13">
         <f t="shared" si="56"/>
-        <v>1869</v>
+        <v>1829</v>
       </c>
       <c r="O295" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29366,7 +29369,7 @@
         <v>18</v>
       </c>
       <c r="C296" s="12" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="D296" s="16" t="s">
         <v>59</v>
@@ -29375,7 +29378,7 @@
         <v>26</v>
       </c>
       <c r="F296" s="12" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="G296" s="13">
         <v>1899</v>
@@ -29437,7 +29440,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="297" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="297" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A297" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
@@ -29446,16 +29449,16 @@
         <v>18</v>
       </c>
       <c r="C297" s="12" t="s">
-        <v>591</v>
-      </c>
-      <c r="D297" s="12" t="s">
-        <v>49</v>
+        <v>587</v>
+      </c>
+      <c r="D297" s="16" t="s">
+        <v>59</v>
       </c>
       <c r="E297" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F297" s="12" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="G297" s="13">
         <v>1899</v>
@@ -29463,7 +29466,7 @@
       <c r="H297" s="13"/>
       <c r="I297" s="13"/>
       <c r="J297" s="13">
-        <v>1899</v>
+        <v>1869</v>
       </c>
       <c r="K297" s="13">
         <f t="shared" si="53"/>
@@ -29479,7 +29482,7 @@
       </c>
       <c r="N297" s="13">
         <f t="shared" si="56"/>
-        <v>1899</v>
+        <v>1869</v>
       </c>
       <c r="O297" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29517,33 +29520,33 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="298" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="298" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A298" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B298" s="12" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C298" s="12" t="s">
-        <v>688</v>
-      </c>
-      <c r="D298" s="16" t="s">
-        <v>71</v>
+        <v>591</v>
+      </c>
+      <c r="D298" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E298" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F298" s="12" t="s">
-        <v>689</v>
+        <v>592</v>
       </c>
       <c r="G298" s="13">
-        <v>1857</v>
+        <v>1899</v>
       </c>
       <c r="H298" s="13"/>
       <c r="I298" s="13"/>
       <c r="J298" s="13">
-        <v>1827</v>
+        <v>1899</v>
       </c>
       <c r="K298" s="13">
         <f t="shared" si="53"/>
@@ -29551,7 +29554,7 @@
       </c>
       <c r="L298" s="13">
         <f t="shared" si="54"/>
-        <v>1857</v>
+        <v>1899</v>
       </c>
       <c r="M298" s="13" t="str">
         <f t="shared" si="55"/>
@@ -29559,7 +29562,7 @@
       </c>
       <c r="N298" s="13">
         <f t="shared" si="56"/>
-        <v>1827</v>
+        <v>1899</v>
       </c>
       <c r="O298" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29603,27 +29606,27 @@
         <v/>
       </c>
       <c r="B299" s="12" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C299" s="12" t="s">
-        <v>593</v>
+        <v>688</v>
       </c>
       <c r="D299" s="16" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E299" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F299" s="12" t="s">
-        <v>594</v>
+        <v>689</v>
       </c>
       <c r="G299" s="13">
-        <v>1900</v>
+        <v>1857</v>
       </c>
       <c r="H299" s="13"/>
       <c r="I299" s="13"/>
       <c r="J299" s="13">
-        <v>1890</v>
+        <v>1827</v>
       </c>
       <c r="K299" s="13">
         <f t="shared" si="53"/>
@@ -29631,7 +29634,7 @@
       </c>
       <c r="L299" s="13">
         <f t="shared" si="54"/>
-        <v>1900</v>
+        <v>1857</v>
       </c>
       <c r="M299" s="13" t="str">
         <f t="shared" si="55"/>
@@ -29639,7 +29642,7 @@
       </c>
       <c r="N299" s="13">
         <f t="shared" si="56"/>
-        <v>1890</v>
+        <v>1827</v>
       </c>
       <c r="O299" s="13" t="str">
         <f t="shared" si="57"/>
@@ -29677,33 +29680,33 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="300" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="300" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A300" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B300" s="12" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C300" s="12" t="s">
-        <v>599</v>
+        <v>593</v>
       </c>
       <c r="D300" s="16" t="s">
         <v>52</v>
       </c>
       <c r="E300" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F300" s="12" t="s">
-        <v>600</v>
+        <v>594</v>
       </c>
       <c r="G300" s="13">
-        <v>1858</v>
+        <v>1900</v>
       </c>
       <c r="H300" s="13"/>
       <c r="I300" s="13"/>
       <c r="J300" s="13">
-        <v>1848</v>
+        <v>1890</v>
       </c>
       <c r="K300" s="13">
         <f t="shared" si="53"/>
@@ -29711,7 +29714,7 @@
       </c>
       <c r="L300" s="13">
         <f t="shared" si="54"/>
-        <v>1858</v>
+        <v>1900</v>
       </c>
       <c r="M300" s="13" t="str">
         <f t="shared" si="55"/>
@@ -29719,7 +29722,7 @@
       </c>
       <c r="N300" s="13">
         <f t="shared" si="56"/>
-        <v>1848</v>
+        <v>1890</v>
       </c>
       <c r="O300" s="13" t="str">
         <f t="shared" si="57"/>
@@ -30477,25 +30480,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="310" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="310" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A310" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B310" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C310" s="12" t="s">
-        <v>624</v>
+        <v>654</v>
       </c>
       <c r="D310" s="16" t="s">
         <v>59</v>
       </c>
       <c r="E310" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F310" s="12" t="s">
-        <v>625</v>
+        <v>655</v>
       </c>
       <c r="G310" s="13">
         <v>1866</v>
@@ -30503,7 +30506,7 @@
       <c r="H310" s="13"/>
       <c r="I310" s="13"/>
       <c r="J310" s="13">
-        <v>1831</v>
+        <v>1846</v>
       </c>
       <c r="K310" s="13">
         <f t="shared" si="53"/>
@@ -30519,7 +30522,7 @@
       </c>
       <c r="N310" s="13">
         <f t="shared" si="56"/>
-        <v>1831</v>
+        <v>1846</v>
       </c>
       <c r="O310" s="13" t="str">
         <f t="shared" si="57"/>
@@ -30557,25 +30560,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="311" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="311" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A311" s="12" t="str">
         <f t="shared" si="52"/>
         <v/>
       </c>
       <c r="B311" s="12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C311" s="12" t="s">
-        <v>654</v>
+        <v>624</v>
       </c>
       <c r="D311" s="16" t="s">
         <v>59</v>
       </c>
       <c r="E311" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F311" s="12" t="s">
-        <v>655</v>
+        <v>625</v>
       </c>
       <c r="G311" s="13">
         <v>1866</v>
@@ -36397,25 +36400,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="384" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="384" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A384" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
       </c>
       <c r="B384" s="12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C384" s="12" t="s">
-        <v>776</v>
-      </c>
-      <c r="D384" s="18" t="s">
-        <v>49</v>
+        <v>817</v>
+      </c>
+      <c r="D384" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E384" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F384" s="12" t="s">
-        <v>777</v>
+        <v>818</v>
       </c>
       <c r="G384" s="13">
         <v>1899</v>
@@ -36477,7 +36480,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="385" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="385" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A385" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
@@ -36486,16 +36489,16 @@
         <v>10</v>
       </c>
       <c r="C385" s="12" t="s">
-        <v>817</v>
+        <v>795</v>
       </c>
       <c r="D385" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E385" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F385" s="12" t="s">
-        <v>818</v>
+        <v>796</v>
       </c>
       <c r="G385" s="13">
         <v>1899</v>
@@ -36557,7 +36560,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="386" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="386" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A386" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
@@ -36566,16 +36569,16 @@
         <v>10</v>
       </c>
       <c r="C386" s="12" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="D386" s="16" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E386" s="12" t="s">
         <v>62</v>
       </c>
       <c r="F386" s="12" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="G386" s="13">
         <v>1899</v>
@@ -36637,25 +36640,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="387" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="387" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A387" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
       </c>
       <c r="B387" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C387" s="12" t="s">
-        <v>799</v>
+        <v>768</v>
       </c>
       <c r="D387" s="16" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E387" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F387" s="12" t="s">
-        <v>800</v>
+        <v>769</v>
       </c>
       <c r="G387" s="13">
         <v>1899</v>
@@ -36663,7 +36666,7 @@
       <c r="H387" s="13"/>
       <c r="I387" s="13"/>
       <c r="J387" s="13">
-        <v>1889</v>
+        <v>1897</v>
       </c>
       <c r="K387" s="13">
         <f t="shared" si="66"/>
@@ -36679,7 +36682,7 @@
       </c>
       <c r="N387" s="13">
         <f t="shared" si="69"/>
-        <v>1889</v>
+        <v>1897</v>
       </c>
       <c r="O387" s="13" t="str">
         <f t="shared" si="70"/>
@@ -36717,25 +36720,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="388" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="388" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A388" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
       </c>
       <c r="B388" s="12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C388" s="12" t="s">
-        <v>768</v>
+        <v>778</v>
       </c>
       <c r="D388" s="16" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E388" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F388" s="12" t="s">
-        <v>769</v>
+        <v>779</v>
       </c>
       <c r="G388" s="13">
         <v>1899</v>
@@ -36743,7 +36746,7 @@
       <c r="H388" s="13"/>
       <c r="I388" s="13"/>
       <c r="J388" s="13">
-        <v>1897</v>
+        <v>1898</v>
       </c>
       <c r="K388" s="13">
         <f t="shared" si="66"/>
@@ -36759,7 +36762,7 @@
       </c>
       <c r="N388" s="13">
         <f t="shared" si="69"/>
-        <v>1897</v>
+        <v>1898</v>
       </c>
       <c r="O388" s="13" t="str">
         <f t="shared" si="70"/>
@@ -36803,19 +36806,19 @@
         <v/>
       </c>
       <c r="B389" s="12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C389" s="12" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="D389" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E389" s="12" t="s">
         <v>62</v>
       </c>
       <c r="F389" s="12" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="G389" s="13">
         <v>1899</v>
@@ -36823,7 +36826,7 @@
       <c r="H389" s="13"/>
       <c r="I389" s="13"/>
       <c r="J389" s="13">
-        <v>1898</v>
+        <v>1899</v>
       </c>
       <c r="K389" s="13">
         <f t="shared" si="66"/>
@@ -36839,7 +36842,7 @@
       </c>
       <c r="N389" s="13">
         <f t="shared" si="69"/>
-        <v>1898</v>
+        <v>1899</v>
       </c>
       <c r="O389" s="13" t="str">
         <f t="shared" si="70"/>
@@ -36877,7 +36880,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="390" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="390" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A390" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
@@ -36886,16 +36889,16 @@
         <v>8</v>
       </c>
       <c r="C390" s="12" t="s">
-        <v>780</v>
-      </c>
-      <c r="D390" s="16" t="s">
-        <v>59</v>
+        <v>782</v>
+      </c>
+      <c r="D390" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E390" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F390" s="12" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="G390" s="13">
         <v>1899</v>
@@ -36957,16 +36960,16 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="391" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="391" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A391" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
       </c>
       <c r="B391" s="12" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C391" s="12" t="s">
-        <v>782</v>
+        <v>710</v>
       </c>
       <c r="D391" s="12" t="s">
         <v>49</v>
@@ -36975,7 +36978,7 @@
         <v>26</v>
       </c>
       <c r="F391" s="12" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="G391" s="13">
         <v>1899</v>
@@ -37046,16 +37049,16 @@
         <v>14</v>
       </c>
       <c r="C392" s="12" t="s">
-        <v>710</v>
-      </c>
-      <c r="D392" s="12" t="s">
-        <v>49</v>
+        <v>868</v>
+      </c>
+      <c r="D392" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E392" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F392" s="12" t="s">
-        <v>784</v>
+        <v>869</v>
       </c>
       <c r="G392" s="13">
         <v>1899</v>
@@ -37126,16 +37129,16 @@
         <v>14</v>
       </c>
       <c r="C393" s="12" t="s">
-        <v>868</v>
-      </c>
-      <c r="D393" s="16" t="s">
-        <v>52</v>
+        <v>863</v>
+      </c>
+      <c r="D393" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E393" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F393" s="12" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="G393" s="13">
         <v>1899</v>
@@ -37197,7 +37200,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="394" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="394" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A394" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
@@ -37206,7 +37209,7 @@
         <v>14</v>
       </c>
       <c r="C394" s="12" t="s">
-        <v>863</v>
+        <v>811</v>
       </c>
       <c r="D394" s="12" t="s">
         <v>49</v>
@@ -37215,7 +37218,7 @@
         <v>62</v>
       </c>
       <c r="F394" s="12" t="s">
-        <v>864</v>
+        <v>812</v>
       </c>
       <c r="G394" s="13">
         <v>1899</v>
@@ -37277,25 +37280,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="395" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="395" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A395" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
       </c>
       <c r="B395" s="12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C395" s="12" t="s">
-        <v>811</v>
-      </c>
-      <c r="D395" s="12" t="s">
+        <v>785</v>
+      </c>
+      <c r="D395" s="18" t="s">
         <v>49</v>
       </c>
       <c r="E395" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F395" s="12" t="s">
-        <v>812</v>
+        <v>786</v>
       </c>
       <c r="G395" s="13">
         <v>1899</v>
@@ -37357,7 +37360,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="396" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="396" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A396" s="12" t="str">
         <f t="shared" si="65"/>
         <v/>
@@ -37366,16 +37369,16 @@
         <v>12</v>
       </c>
       <c r="C396" s="12" t="s">
-        <v>785</v>
-      </c>
-      <c r="D396" s="18" t="s">
-        <v>49</v>
+        <v>787</v>
+      </c>
+      <c r="D396" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E396" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F396" s="12" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="G396" s="13">
         <v>1899</v>
@@ -37446,16 +37449,16 @@
         <v>12</v>
       </c>
       <c r="C397" s="12" t="s">
-        <v>787</v>
-      </c>
-      <c r="D397" s="16" t="s">
-        <v>52</v>
+        <v>776</v>
+      </c>
+      <c r="D397" s="18" t="s">
+        <v>49</v>
       </c>
       <c r="E397" s="12" t="s">
         <v>62</v>
       </c>
       <c r="F397" s="12" t="s">
-        <v>788</v>
+        <v>777</v>
       </c>
       <c r="G397" s="13">
         <v>1899</v>
@@ -56945,19 +56948,19 @@
         <v/>
       </c>
       <c r="B646" s="12" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C646" s="12" t="s">
-        <v>1251</v>
-      </c>
-      <c r="D646" s="16" t="s">
-        <v>71</v>
+        <v>1281</v>
+      </c>
+      <c r="D646" s="12" t="s">
+        <v>304</v>
       </c>
       <c r="E646" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F646" s="12" t="s">
-        <v>1252</v>
+        <v>1282</v>
       </c>
       <c r="G646" s="13">
         <v>1845</v>
@@ -57023,19 +57026,19 @@
         <v/>
       </c>
       <c r="B647" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C647" s="12" t="s">
-        <v>1281</v>
-      </c>
-      <c r="D647" s="12" t="s">
-        <v>304</v>
+        <v>1237</v>
+      </c>
+      <c r="D647" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E647" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F647" s="12" t="s">
-        <v>1282</v>
+        <v>1238</v>
       </c>
       <c r="G647" s="13">
         <v>1845</v>
@@ -57043,7 +57046,7 @@
       <c r="H647" s="13"/>
       <c r="I647" s="13"/>
       <c r="J647" s="13">
-        <v>1834</v>
+        <v>1835</v>
       </c>
       <c r="K647" s="13">
         <f t="shared" si="118"/>
@@ -57059,7 +57062,7 @@
       </c>
       <c r="N647" s="13">
         <f t="shared" si="121"/>
-        <v>1834</v>
+        <v>1835</v>
       </c>
       <c r="O647" s="13" t="str">
         <f t="shared" si="122"/>
@@ -57095,7 +57098,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="648" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="648" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A648" s="12" t="str">
         <f t="shared" si="117"/>
         <v/>
@@ -57104,7 +57107,7 @@
         <v>12</v>
       </c>
       <c r="C648" s="12" t="s">
-        <v>1237</v>
+        <v>1239</v>
       </c>
       <c r="D648" s="16" t="s">
         <v>52</v>
@@ -57113,7 +57116,7 @@
         <v>26</v>
       </c>
       <c r="F648" s="12" t="s">
-        <v>1238</v>
+        <v>1240</v>
       </c>
       <c r="G648" s="13">
         <v>1845</v>
@@ -57173,25 +57176,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="649" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="649" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A649" s="12" t="str">
         <f t="shared" si="117"/>
         <v/>
       </c>
       <c r="B649" s="12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C649" s="12" t="s">
-        <v>1239</v>
+        <v>1243</v>
       </c>
       <c r="D649" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E649" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F649" s="12" t="s">
-        <v>1240</v>
+        <v>1244</v>
       </c>
       <c r="G649" s="13">
         <v>1845</v>
@@ -57199,7 +57202,7 @@
       <c r="H649" s="13"/>
       <c r="I649" s="13"/>
       <c r="J649" s="13">
-        <v>1835</v>
+        <v>1839</v>
       </c>
       <c r="K649" s="13">
         <f t="shared" si="118"/>
@@ -57215,7 +57218,7 @@
       </c>
       <c r="N649" s="13">
         <f t="shared" si="121"/>
-        <v>1835</v>
+        <v>1839</v>
       </c>
       <c r="O649" s="13" t="str">
         <f t="shared" si="122"/>
@@ -57251,25 +57254,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="650" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="650" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A650" s="12" t="str">
         <f t="shared" si="117"/>
         <v/>
       </c>
       <c r="B650" s="12" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C650" s="12" t="s">
-        <v>1243</v>
-      </c>
-      <c r="D650" s="16" t="s">
-        <v>59</v>
+        <v>1497</v>
+      </c>
+      <c r="D650" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E650" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F650" s="12" t="s">
-        <v>1244</v>
+        <v>1498</v>
       </c>
       <c r="G650" s="13">
         <v>1845</v>
@@ -57277,7 +57280,7 @@
       <c r="H650" s="13"/>
       <c r="I650" s="13"/>
       <c r="J650" s="13">
-        <v>1839</v>
+        <v>1845</v>
       </c>
       <c r="K650" s="13">
         <f t="shared" si="118"/>
@@ -57293,7 +57296,7 @@
       </c>
       <c r="N650" s="13">
         <f t="shared" si="121"/>
-        <v>1839</v>
+        <v>1845</v>
       </c>
       <c r="O650" s="13" t="str">
         <f t="shared" si="122"/>
@@ -57335,19 +57338,19 @@
         <v/>
       </c>
       <c r="B651" s="12" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C651" s="12" t="s">
-        <v>1497</v>
+        <v>1249</v>
       </c>
       <c r="D651" s="12" t="s">
-        <v>49</v>
+        <v>749</v>
       </c>
       <c r="E651" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F651" s="12" t="s">
-        <v>1498</v>
+        <v>1250</v>
       </c>
       <c r="G651" s="13">
         <v>1845</v>
@@ -57413,19 +57416,19 @@
         <v/>
       </c>
       <c r="B652" s="12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C652" s="12" t="s">
-        <v>1249</v>
-      </c>
-      <c r="D652" s="12" t="s">
-        <v>749</v>
+        <v>1251</v>
+      </c>
+      <c r="D652" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="E652" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F652" s="12" t="s">
-        <v>1250</v>
+        <v>1252</v>
       </c>
       <c r="G652" s="13">
         <v>1845</v>
@@ -57433,7 +57436,7 @@
       <c r="H652" s="13"/>
       <c r="I652" s="13"/>
       <c r="J652" s="13">
-        <v>1845</v>
+        <v>1849</v>
       </c>
       <c r="K652" s="13">
         <f t="shared" si="118"/>
@@ -57449,7 +57452,7 @@
       </c>
       <c r="N652" s="13">
         <f t="shared" si="121"/>
-        <v>1845</v>
+        <v>1849</v>
       </c>
       <c r="O652" s="13" t="str">
         <f t="shared" si="122"/>
@@ -57641,7 +57644,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="655" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="655" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
       <c r="A655" s="12" t="str">
         <f t="shared" ref="A655:A718" si="130">IF($T655="","",1+COUNTIF($W$15:$W$878,"&lt;"&amp;W655))</f>
         <v/>
@@ -57650,16 +57653,16 @@
         <v>10</v>
       </c>
       <c r="C655" s="12" t="s">
-        <v>1261</v>
+        <v>1389</v>
       </c>
       <c r="D655" s="16" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E655" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F655" s="12" t="s">
-        <v>1262</v>
+        <v>1390</v>
       </c>
       <c r="G655" s="13">
         <v>1848</v>
@@ -57667,7 +57670,7 @@
       <c r="H655" s="13"/>
       <c r="I655" s="13"/>
       <c r="J655" s="13">
-        <v>1818</v>
+        <v>1819</v>
       </c>
       <c r="K655" s="13">
         <f t="shared" ref="K655:K684" si="131">IF(AND(IFERROR(SEARCH("현대오일뱅크",$C655),0)&gt;0,IFERROR(SEARCH("직영",$C655),0)&gt;0),$B$13,0)</f>
@@ -57683,7 +57686,7 @@
       </c>
       <c r="N655" s="13">
         <f t="shared" ref="N655:N718" si="134">IF($J655="","",$J655+$K655)</f>
-        <v>1818</v>
+        <v>1819</v>
       </c>
       <c r="O655" s="13" t="str">
         <f t="shared" ref="O655:O718" si="135">IF($B$10=0,"",IFERROR(IF($B$4&gt;0,"휘발유 "&amp;TEXT(IF($L655="",1/0,$L655*$B$4),"#,##0")&amp;"원","")&amp;IF($B$5&gt;0,IF($B$4&gt;0," / ","")&amp;"고급유 "&amp;TEXT(IF($M655="",1/0,$M655*$B$5),"#,##0")&amp;"원","")&amp;IF($B$6&gt;0,IF(OR($B$4&gt;0,$B$5&gt;0)," / ","")&amp;"경유 "&amp;TEXT(IF($N655="",1/0,$N655*$B$6),"#,##0")&amp;"원",""),""))</f>
@@ -57719,7 +57722,7 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="656" spans="1:23" s="8" customFormat="1" ht="28.5" customHeight="1">
+    <row r="656" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A656" s="12" t="str">
         <f t="shared" si="130"/>
         <v/>
@@ -57728,16 +57731,16 @@
         <v>10</v>
       </c>
       <c r="C656" s="12" t="s">
-        <v>1389</v>
-      </c>
-      <c r="D656" s="16" t="s">
-        <v>52</v>
+        <v>1429</v>
+      </c>
+      <c r="D656" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E656" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F656" s="12" t="s">
-        <v>1390</v>
+        <v>1430</v>
       </c>
       <c r="G656" s="13">
         <v>1848</v>
@@ -57803,19 +57806,19 @@
         <v/>
       </c>
       <c r="B657" s="12" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C657" s="12" t="s">
-        <v>1429</v>
-      </c>
-      <c r="D657" s="12" t="s">
-        <v>49</v>
+        <v>1453</v>
+      </c>
+      <c r="D657" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="E657" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F657" s="12" t="s">
-        <v>1430</v>
+        <v>1454</v>
       </c>
       <c r="G657" s="13">
         <v>1848</v>
@@ -57823,7 +57826,7 @@
       <c r="H657" s="13"/>
       <c r="I657" s="13"/>
       <c r="J657" s="13">
-        <v>1819</v>
+        <v>1824</v>
       </c>
       <c r="K657" s="13">
         <f t="shared" si="131"/>
@@ -57839,7 +57842,7 @@
       </c>
       <c r="N657" s="13">
         <f t="shared" si="134"/>
-        <v>1819</v>
+        <v>1824</v>
       </c>
       <c r="O657" s="13" t="str">
         <f t="shared" si="135"/>
@@ -57881,19 +57884,19 @@
         <v/>
       </c>
       <c r="B658" s="12" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C658" s="12" t="s">
-        <v>1453</v>
+        <v>1261</v>
       </c>
       <c r="D658" s="16" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E658" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F658" s="12" t="s">
-        <v>1454</v>
+        <v>1262</v>
       </c>
       <c r="G658" s="13">
         <v>1848</v>
@@ -57901,7 +57904,7 @@
       <c r="H658" s="13"/>
       <c r="I658" s="13"/>
       <c r="J658" s="13">
-        <v>1824</v>
+        <v>1848</v>
       </c>
       <c r="K658" s="13">
         <f t="shared" si="131"/>
@@ -57917,7 +57920,7 @@
       </c>
       <c r="N658" s="13">
         <f t="shared" si="134"/>
-        <v>1824</v>
+        <v>1848</v>
       </c>
       <c r="O658" s="13" t="str">
         <f t="shared" si="135"/>
@@ -57959,19 +57962,19 @@
         <v/>
       </c>
       <c r="B659" s="12" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C659" s="12" t="s">
-        <v>1491</v>
-      </c>
-      <c r="D659" s="16" t="s">
-        <v>52</v>
+        <v>1263</v>
+      </c>
+      <c r="D659" s="18" t="s">
+        <v>749</v>
       </c>
       <c r="E659" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F659" s="12" t="s">
-        <v>1492</v>
+        <v>1264</v>
       </c>
       <c r="G659" s="13">
         <v>1848</v>
@@ -57979,7 +57982,7 @@
       <c r="H659" s="13"/>
       <c r="I659" s="13"/>
       <c r="J659" s="13">
-        <v>1834</v>
+        <v>1855</v>
       </c>
       <c r="K659" s="13">
         <f t="shared" si="131"/>
@@ -57995,7 +57998,7 @@
       </c>
       <c r="N659" s="13">
         <f t="shared" si="134"/>
-        <v>1834</v>
+        <v>1855</v>
       </c>
       <c r="O659" s="13" t="str">
         <f t="shared" si="135"/>
@@ -58037,19 +58040,19 @@
         <v/>
       </c>
       <c r="B660" s="12" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C660" s="12" t="s">
-        <v>1263</v>
-      </c>
-      <c r="D660" s="18" t="s">
-        <v>749</v>
+        <v>1491</v>
+      </c>
+      <c r="D660" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="E660" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F660" s="12" t="s">
-        <v>1264</v>
+        <v>1492</v>
       </c>
       <c r="G660" s="13">
         <v>1848</v>
@@ -58057,7 +58060,7 @@
       <c r="H660" s="13"/>
       <c r="I660" s="13"/>
       <c r="J660" s="13">
-        <v>1855</v>
+        <v>1884</v>
       </c>
       <c r="K660" s="13">
         <f t="shared" si="131"/>
@@ -58073,7 +58076,7 @@
       </c>
       <c r="N660" s="13">
         <f t="shared" si="134"/>
-        <v>1855</v>
+        <v>1884</v>
       </c>
       <c r="O660" s="13" t="str">
         <f t="shared" si="135"/>
@@ -73236,25 +73239,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="855" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
+    <row r="855" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
       <c r="A855" s="12" t="str">
         <f t="shared" si="174"/>
         <v/>
       </c>
       <c r="B855" s="12" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C855" s="12" t="s">
-        <v>1693</v>
+        <v>1695</v>
       </c>
       <c r="D855" s="16" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E855" s="12" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="F855" s="12" t="s">
-        <v>1694</v>
+        <v>1696</v>
       </c>
       <c r="G855" s="13">
         <v>1909</v>
@@ -73262,7 +73265,7 @@
       <c r="H855" s="13"/>
       <c r="I855" s="13"/>
       <c r="J855" s="13">
-        <v>1899</v>
+        <v>1890</v>
       </c>
       <c r="K855" s="13">
         <f t="shared" si="173"/>
@@ -73278,7 +73281,7 @@
       </c>
       <c r="N855" s="13">
         <f t="shared" si="177"/>
-        <v>1899</v>
+        <v>1890</v>
       </c>
       <c r="O855" s="13" t="str">
         <f t="shared" si="178"/>
@@ -73314,25 +73317,25 @@
         <v>1000000000000000</v>
       </c>
     </row>
-    <row r="856" spans="1:23" s="17" customFormat="1" ht="28.5" customHeight="1">
+    <row r="856" spans="1:23" s="2" customFormat="1" ht="28.5" customHeight="1">
       <c r="A856" s="12" t="str">
         <f t="shared" si="174"/>
         <v/>
       </c>
       <c r="B856" s="12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C856" s="12" t="s">
-        <v>1695</v>
+        <v>1693</v>
       </c>
       <c r="D856" s="16" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E856" s="12" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="F856" s="12" t="s">
-        <v>1696</v>
+        <v>1694</v>
       </c>
       <c r="G856" s="13">
         <v>1909</v>
@@ -75213,199 +75216,528 @@
       </c>
     </row>
     <row r="4" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A4" s="21"/>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
+      <c r="A4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E4" s="23">
+        <v>1886</v>
+      </c>
+      <c r="F4" s="23">
+        <v>1896</v>
+      </c>
+      <c r="G4" s="23">
+        <f t="shared" ref="G4:G16" si="0">IF(OR(E4="",F4=""),"",F4-E4)</f>
+        <v>10</v>
+      </c>
+      <c r="H4" s="23">
+        <v>2250</v>
+      </c>
+      <c r="I4" s="23">
+        <v>2250</v>
+      </c>
+      <c r="J4" s="23">
+        <f t="shared" ref="J4:J16" si="1">IF(OR(H4="",I4=""),"",I4-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="23">
+        <v>1876</v>
+      </c>
+      <c r="L4" s="23">
+        <v>1876</v>
+      </c>
+      <c r="M4" s="23">
+        <f t="shared" ref="M4:M16" si="2">IF(OR(K4="",L4=""),"",L4-K4)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A5" s="21"/>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
+      <c r="A5" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>470</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>471</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E5" s="23">
+        <v>1859</v>
+      </c>
+      <c r="F5" s="23">
+        <v>1859</v>
+      </c>
+      <c r="G5" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H5" s="23"/>
       <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
+      <c r="J5" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K5" s="23">
+        <v>1849</v>
+      </c>
+      <c r="L5" s="23">
+        <v>1869</v>
+      </c>
+      <c r="M5" s="23">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
     </row>
     <row r="6" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A6" s="21"/>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
+      <c r="A6" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>436</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>437</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E6" s="23">
+        <v>1869</v>
+      </c>
+      <c r="F6" s="23">
+        <v>1869</v>
+      </c>
+      <c r="G6" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H6" s="23"/>
       <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
+      <c r="J6" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K6" s="23">
+        <v>1849</v>
+      </c>
+      <c r="L6" s="23">
+        <v>1854</v>
+      </c>
+      <c r="M6" s="23">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
     </row>
     <row r="7" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A7" s="21"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
+      <c r="A7" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>474</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>475</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E7" s="23">
+        <v>1880</v>
+      </c>
+      <c r="F7" s="23">
+        <v>1880</v>
+      </c>
+      <c r="G7" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H7" s="23"/>
       <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
+      <c r="J7" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K7" s="23">
+        <v>1860</v>
+      </c>
+      <c r="L7" s="23">
+        <v>1890</v>
+      </c>
+      <c r="M7" s="23">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
     </row>
     <row r="8" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A8" s="21"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
+      <c r="A8" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>523</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>524</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E8" s="23">
+        <v>1889</v>
+      </c>
+      <c r="F8" s="23">
+        <v>1889</v>
+      </c>
+      <c r="G8" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H8" s="23"/>
       <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
+      <c r="J8" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K8" s="23">
+        <v>1847</v>
+      </c>
+      <c r="L8" s="23">
+        <v>1867</v>
+      </c>
+      <c r="M8" s="23">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
     </row>
     <row r="9" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A9" s="21"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
+      <c r="A9" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>571</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>572</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E9" s="23">
+        <v>1854</v>
+      </c>
+      <c r="F9" s="23">
+        <v>1854</v>
+      </c>
+      <c r="G9" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H9" s="23"/>
       <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
+      <c r="J9" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K9" s="23">
+        <v>1837</v>
+      </c>
+      <c r="L9" s="23">
+        <v>1829</v>
+      </c>
+      <c r="M9" s="23">
+        <f t="shared" si="2"/>
+        <v>-8</v>
+      </c>
     </row>
     <row r="10" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A10" s="21"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
+      <c r="A10" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>599</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>600</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E10" s="23">
+        <v>1858</v>
+      </c>
+      <c r="F10" s="23">
+        <v>1848</v>
+      </c>
+      <c r="G10" s="23">
+        <f t="shared" si="0"/>
+        <v>-10</v>
+      </c>
       <c r="H10" s="23"/>
       <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
+      <c r="J10" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K10" s="23">
+        <v>1848</v>
+      </c>
+      <c r="L10" s="23">
+        <v>1838</v>
+      </c>
+      <c r="M10" s="23">
+        <f t="shared" si="2"/>
+        <v>-10</v>
+      </c>
     </row>
     <row r="11" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A11" s="21"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
+      <c r="A11" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>624</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>625</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E11" s="23">
+        <v>1866</v>
+      </c>
+      <c r="F11" s="23">
+        <v>1866</v>
+      </c>
+      <c r="G11" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H11" s="23"/>
       <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
+      <c r="J11" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K11" s="23">
+        <v>1831</v>
+      </c>
+      <c r="L11" s="23">
+        <v>1846</v>
+      </c>
+      <c r="M11" s="23">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A12" s="21"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
+      <c r="A12" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>776</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>777</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E12" s="23">
+        <v>1899</v>
+      </c>
+      <c r="F12" s="23">
+        <v>1899</v>
+      </c>
+      <c r="G12" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H12" s="23"/>
       <c r="I12" s="23"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="23"/>
-      <c r="M12" s="23"/>
+      <c r="J12" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K12" s="23">
+        <v>1889</v>
+      </c>
+      <c r="L12" s="23">
+        <v>1899</v>
+      </c>
+      <c r="M12" s="23">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
     </row>
     <row r="13" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A13" s="21"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
+      <c r="A13" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E13" s="23">
+        <v>1845</v>
+      </c>
+      <c r="F13" s="23">
+        <v>1845</v>
+      </c>
+      <c r="G13" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H13" s="23"/>
       <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="23"/>
+      <c r="J13" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K13" s="23">
+        <v>1834</v>
+      </c>
+      <c r="L13" s="23">
+        <v>1849</v>
+      </c>
+      <c r="M13" s="23">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A14" s="21"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
+      <c r="A14" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>1262</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E14" s="23">
+        <v>1848</v>
+      </c>
+      <c r="F14" s="23">
+        <v>1848</v>
+      </c>
+      <c r="G14" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H14" s="23"/>
       <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
+      <c r="J14" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K14" s="23">
+        <v>1818</v>
+      </c>
+      <c r="L14" s="23">
+        <v>1848</v>
+      </c>
+      <c r="M14" s="23">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
     </row>
     <row r="15" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A15" s="21"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
+      <c r="A15" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>1492</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E15" s="23">
+        <v>1848</v>
+      </c>
+      <c r="F15" s="23">
+        <v>1848</v>
+      </c>
+      <c r="G15" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H15" s="23"/>
       <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
+      <c r="J15" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K15" s="23">
+        <v>1834</v>
+      </c>
+      <c r="L15" s="23">
+        <v>1884</v>
+      </c>
+      <c r="M15" s="23">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
     </row>
     <row r="16" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A16" s="21"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
+      <c r="A16" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>1695</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>1696</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E16" s="23">
+        <v>1909</v>
+      </c>
+      <c r="F16" s="23">
+        <v>1909</v>
+      </c>
+      <c r="G16" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="H16" s="23"/>
       <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
+      <c r="J16" s="23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K16" s="23">
+        <v>1899</v>
+      </c>
+      <c r="L16" s="23">
+        <v>1890</v>
+      </c>
+      <c r="M16" s="23">
+        <f t="shared" si="2"/>
+        <v>-9</v>
+      </c>
     </row>
     <row r="17" spans="1:13" s="17" customFormat="1" ht="25.5" customHeight="1">
       <c r="A17" s="21"/>
@@ -78817,7 +79149,7 @@
     <mergeCell ref="A1:M1"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
-  <conditionalFormatting sqref="G4:G4">
+  <conditionalFormatting sqref="G4:G16">
     <cfRule type="cellIs" dxfId="5" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
@@ -78825,7 +79157,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J4:J4">
+  <conditionalFormatting sqref="J4:J16">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
@@ -78833,7 +79165,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M4:M4">
+  <conditionalFormatting sqref="M4:M16">
     <cfRule type="cellIs" dxfId="1" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Simplify buffer reservation and workbook parsing
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4833" uniqueCount="1767">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4697" uniqueCount="1764">
   <si>
     <t>유류비 계산(혼유, 지역화폐 등)</t>
   </si>
@@ -5136,9 +5136,6 @@
     <t>충북 청주시 흥덕구 엘지로 11</t>
   </si>
   <si>
-    <t>세종시 부강면 시목부강로 423</t>
-  </si>
-  <si>
     <t>충북 청주시 청원구 오창읍 두릉유리로 204</t>
   </si>
   <si>
@@ -5389,12 +5386,6 @@
   </si>
   <si>
     <t>현행화 일자: 2026-09-03</t>
-  </si>
-  <si>
-    <t>가격변동</t>
-  </si>
-  <si>
-    <t>폐업</t>
   </si>
 </sst>
 </file>
@@ -9821,7 +9812,7 @@
         <v>10</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>1753</v>
+        <v>1752</v>
       </c>
       <c r="D52" s="11" t="s">
         <v>45</v>
@@ -9830,7 +9821,7 @@
         <v>26</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>1754</v>
+        <v>1753</v>
       </c>
       <c r="G52" s="12">
         <v>1827</v>
@@ -10221,7 +10212,7 @@
         <v>6</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>1713</v>
+        <v>1712</v>
       </c>
       <c r="D57" s="15" t="s">
         <v>45</v>
@@ -10230,7 +10221,7 @@
         <v>26</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="G57" s="12">
         <v>1825</v>
@@ -13903,7 +13894,7 @@
         <v>6</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="D103" s="15" t="s">
         <v>45</v>
@@ -13912,7 +13903,7 @@
         <v>26</v>
       </c>
       <c r="F103" s="11" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="G103" s="12">
         <v>1822</v>
@@ -17587,7 +17578,7 @@
         <v>6</v>
       </c>
       <c r="C149" s="11" t="s">
-        <v>1698</v>
+        <v>1697</v>
       </c>
       <c r="D149" s="15" t="s">
         <v>45</v>
@@ -17596,7 +17587,7 @@
         <v>61</v>
       </c>
       <c r="F149" s="11" t="s">
-        <v>1699</v>
+        <v>1698</v>
       </c>
       <c r="G149" s="12">
         <v>1866</v>
@@ -18951,7 +18942,7 @@
         <v>14</v>
       </c>
       <c r="C166" s="11" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
       <c r="D166" s="15" t="s">
         <v>80</v>
@@ -18960,7 +18951,7 @@
         <v>26</v>
       </c>
       <c r="F166" s="11" t="s">
-        <v>1712</v>
+        <v>1711</v>
       </c>
       <c r="G166" s="12">
         <v>1859</v>
@@ -20315,7 +20306,7 @@
         <v>16</v>
       </c>
       <c r="C183" s="11" t="s">
-        <v>1686</v>
+        <v>1685</v>
       </c>
       <c r="D183" s="15" t="s">
         <v>45</v>
@@ -20324,7 +20315,7 @@
         <v>26</v>
       </c>
       <c r="F183" s="11" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="G183" s="12">
         <v>1830</v>
@@ -24795,7 +24786,7 @@
         <v>6</v>
       </c>
       <c r="C239" s="11" t="s">
-        <v>1688</v>
+        <v>1687</v>
       </c>
       <c r="D239" s="15" t="s">
         <v>45</v>
@@ -24804,7 +24795,7 @@
         <v>26</v>
       </c>
       <c r="F239" s="11" t="s">
-        <v>1689</v>
+        <v>1688</v>
       </c>
       <c r="G239" s="12">
         <v>1829</v>
@@ -26635,7 +26626,7 @@
         <v>16</v>
       </c>
       <c r="C262" s="11" t="s">
-        <v>1730</v>
+        <v>1729</v>
       </c>
       <c r="D262" s="15" t="s">
         <v>80</v>
@@ -26644,7 +26635,7 @@
         <v>61</v>
       </c>
       <c r="F262" s="11" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="G262" s="12">
         <v>1880</v>
@@ -27115,7 +27106,7 @@
         <v>10</v>
       </c>
       <c r="C268" s="11" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="D268" s="15" t="s">
         <v>80</v>
@@ -27124,7 +27115,7 @@
         <v>61</v>
       </c>
       <c r="F268" s="11" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="G268" s="12">
         <v>1839</v>
@@ -27195,7 +27186,7 @@
         <v>10</v>
       </c>
       <c r="C269" s="11" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="D269" s="15" t="s">
         <v>45</v>
@@ -27204,7 +27195,7 @@
         <v>26</v>
       </c>
       <c r="F269" s="11" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="G269" s="12">
         <v>1839</v>
@@ -27355,7 +27346,7 @@
         <v>10</v>
       </c>
       <c r="C271" s="11" t="s">
-        <v>1684</v>
+        <v>1683</v>
       </c>
       <c r="D271" s="11" t="s">
         <v>57</v>
@@ -27364,7 +27355,7 @@
         <v>26</v>
       </c>
       <c r="F271" s="11" t="s">
-        <v>1685</v>
+        <v>1684</v>
       </c>
       <c r="G271" s="12">
         <v>1844</v>
@@ -28155,7 +28146,7 @@
         <v>18</v>
       </c>
       <c r="C281" s="11" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
       <c r="D281" s="15" t="s">
         <v>45</v>
@@ -28164,7 +28155,7 @@
         <v>61</v>
       </c>
       <c r="F281" s="11" t="s">
-        <v>1691</v>
+        <v>1690</v>
       </c>
       <c r="G281" s="12">
         <v>1890</v>
@@ -29355,7 +29346,7 @@
         <v>8</v>
       </c>
       <c r="C296" s="11" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="D296" s="11" t="s">
         <v>57</v>
@@ -29364,7 +29355,7 @@
         <v>26</v>
       </c>
       <c r="F296" s="11" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="G296" s="12">
         <v>1855</v>
@@ -29435,7 +29426,7 @@
         <v>8</v>
       </c>
       <c r="C297" s="11" t="s">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="D297" s="15" t="s">
         <v>60</v>
@@ -29444,7 +29435,7 @@
         <v>26</v>
       </c>
       <c r="F297" s="11" t="s">
-        <v>1737</v>
+        <v>1736</v>
       </c>
       <c r="G297" s="12">
         <v>1855</v>
@@ -29915,7 +29906,7 @@
         <v>18</v>
       </c>
       <c r="C303" s="11" t="s">
-        <v>1704</v>
+        <v>1703</v>
       </c>
       <c r="D303" s="11" t="s">
         <v>57</v>
@@ -29924,7 +29915,7 @@
         <v>61</v>
       </c>
       <c r="F303" s="11" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="G303" s="12">
         <v>1899</v>
@@ -32635,7 +32626,7 @@
         <v>8</v>
       </c>
       <c r="C337" s="11" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="D337" s="15" t="s">
         <v>45</v>
@@ -32644,7 +32635,7 @@
         <v>61</v>
       </c>
       <c r="F337" s="11" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="G337" s="12">
         <v>1875</v>
@@ -34235,7 +34226,7 @@
         <v>14</v>
       </c>
       <c r="C357" s="11" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="D357" s="15" t="s">
         <v>45</v>
@@ -34244,7 +34235,7 @@
         <v>26</v>
       </c>
       <c r="F357" s="11" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="G357" s="12">
         <v>1889</v>
@@ -34395,7 +34386,7 @@
         <v>10</v>
       </c>
       <c r="C359" s="11" t="s">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="D359" s="15" t="s">
         <v>45</v>
@@ -34404,7 +34395,7 @@
         <v>26</v>
       </c>
       <c r="F359" s="11" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="G359" s="12">
         <v>1890</v>
@@ -36635,7 +36626,7 @@
         <v>10</v>
       </c>
       <c r="C387" s="11" t="s">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="D387" s="11" t="s">
         <v>57</v>
@@ -36644,7 +36635,7 @@
         <v>26</v>
       </c>
       <c r="F387" s="11" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="G387" s="12">
         <v>1898</v>
@@ -37195,7 +37186,7 @@
         <v>14</v>
       </c>
       <c r="C394" s="11" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
       <c r="D394" s="11" t="s">
         <v>57</v>
@@ -37204,7 +37195,7 @@
         <v>61</v>
       </c>
       <c r="F394" s="11" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="G394" s="12">
         <v>1899</v>
@@ -40075,7 +40066,7 @@
         <v>12</v>
       </c>
       <c r="C430" s="11" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="D430" s="15" t="s">
         <v>60</v>
@@ -40084,7 +40075,7 @@
         <v>61</v>
       </c>
       <c r="F430" s="11" t="s">
-        <v>1708</v>
+        <v>1707</v>
       </c>
       <c r="G430" s="12">
         <v>1960</v>
@@ -41017,7 +41008,7 @@
         <v>12</v>
       </c>
       <c r="C442" s="11" t="s">
-        <v>1757</v>
+        <v>1756</v>
       </c>
       <c r="D442" s="11" t="s">
         <v>104</v>
@@ -41026,7 +41017,7 @@
         <v>26</v>
       </c>
       <c r="F442" s="11" t="s">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="G442" s="12">
         <v>1799</v>
@@ -42345,7 +42336,7 @@
         <v>14</v>
       </c>
       <c r="C459" s="11" t="s">
-        <v>1740</v>
+        <v>1739</v>
       </c>
       <c r="D459" s="15" t="s">
         <v>45</v>
@@ -42354,7 +42345,7 @@
         <v>26</v>
       </c>
       <c r="F459" s="11" t="s">
-        <v>1741</v>
+        <v>1740</v>
       </c>
       <c r="G459" s="12">
         <v>1809</v>
@@ -48039,7 +48030,7 @@
         <v>10</v>
       </c>
       <c r="C532" s="11" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="D532" s="15" t="s">
         <v>80</v>
@@ -48048,7 +48039,7 @@
         <v>26</v>
       </c>
       <c r="F532" s="11" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="G532" s="12">
         <v>1819</v>
@@ -48819,7 +48810,7 @@
         <v>10</v>
       </c>
       <c r="C542" s="11" t="s">
-        <v>1762</v>
+        <v>1761</v>
       </c>
       <c r="D542" s="11" t="s">
         <v>48</v>
@@ -48828,7 +48819,7 @@
         <v>26</v>
       </c>
       <c r="F542" s="11" t="s">
-        <v>1763</v>
+        <v>1762</v>
       </c>
       <c r="G542" s="12">
         <v>1823</v>
@@ -50379,7 +50370,7 @@
         <v>10</v>
       </c>
       <c r="C562" s="11" t="s">
-        <v>1759</v>
+        <v>1758</v>
       </c>
       <c r="D562" s="11" t="s">
         <v>57</v>
@@ -51393,7 +51384,7 @@
         <v>12</v>
       </c>
       <c r="C575" s="11" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="D575" s="15" t="s">
         <v>45</v>
@@ -51402,7 +51393,7 @@
         <v>26</v>
       </c>
       <c r="F575" s="11" t="s">
-        <v>1733</v>
+        <v>1732</v>
       </c>
       <c r="G575" s="12">
         <v>1825</v>
@@ -52017,7 +52008,7 @@
         <v>6</v>
       </c>
       <c r="C583" s="11" t="s">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="D583" s="11" t="s">
         <v>45</v>
@@ -52026,7 +52017,7 @@
         <v>26</v>
       </c>
       <c r="F583" s="11" t="s">
-        <v>1761</v>
+        <v>1760</v>
       </c>
       <c r="G583" s="12">
         <v>1828</v>
@@ -52494,7 +52485,7 @@
         <v>61</v>
       </c>
       <c r="F589" s="11" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="G589" s="12">
         <v>1828</v>
@@ -54435,7 +54426,7 @@
         <v>10</v>
       </c>
       <c r="C614" s="11" t="s">
-        <v>1700</v>
+        <v>1699</v>
       </c>
       <c r="D614" s="15" t="s">
         <v>45</v>
@@ -54444,7 +54435,7 @@
         <v>26</v>
       </c>
       <c r="F614" s="11" t="s">
-        <v>1701</v>
+        <v>1700</v>
       </c>
       <c r="G614" s="12">
         <v>1829</v>
@@ -57711,7 +57702,7 @@
         <v>10</v>
       </c>
       <c r="C656" s="11" t="s">
-        <v>1738</v>
+        <v>1737</v>
       </c>
       <c r="D656" s="15" t="s">
         <v>45</v>
@@ -57720,7 +57711,7 @@
         <v>61</v>
       </c>
       <c r="F656" s="11" t="s">
-        <v>1739</v>
+        <v>1738</v>
       </c>
       <c r="G656" s="12">
         <v>1839</v>
@@ -64652,7 +64643,7 @@
         <v>12</v>
       </c>
       <c r="C745" s="11" t="s">
-        <v>1694</v>
+        <v>1693</v>
       </c>
       <c r="D745" s="15" t="s">
         <v>45</v>
@@ -64661,7 +64652,7 @@
         <v>61</v>
       </c>
       <c r="F745" s="11" t="s">
-        <v>1695</v>
+        <v>1694</v>
       </c>
       <c r="G745" s="12">
         <v>1856</v>
@@ -66523,7 +66514,7 @@
         <v>6</v>
       </c>
       <c r="C769" s="11" t="s">
-        <v>1696</v>
+        <v>1695</v>
       </c>
       <c r="D769" s="15" t="s">
         <v>45</v>
@@ -66532,7 +66523,7 @@
         <v>61</v>
       </c>
       <c r="F769" s="11" t="s">
-        <v>1697</v>
+        <v>1696</v>
       </c>
       <c r="G769" s="12">
         <v>1866</v>
@@ -67380,7 +67371,7 @@
         <v>12</v>
       </c>
       <c r="C780" s="11" t="s">
-        <v>1717</v>
+        <v>1716</v>
       </c>
       <c r="D780" s="15" t="s">
         <v>80</v>
@@ -67389,7 +67380,7 @@
         <v>26</v>
       </c>
       <c r="F780" s="11" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="G780" s="12">
         <v>1869</v>
@@ -71510,7 +71501,7 @@
         <v>16</v>
       </c>
       <c r="C833" s="11" t="s">
-        <v>1755</v>
+        <v>1754</v>
       </c>
       <c r="D833" s="11" t="s">
         <v>57</v>
@@ -71519,7 +71510,7 @@
         <v>26</v>
       </c>
       <c r="F833" s="11" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="G833" s="12">
         <v>1895</v>
@@ -71744,7 +71735,7 @@
         <v>10</v>
       </c>
       <c r="C836" s="11" t="s">
-        <v>1702</v>
+        <v>1701</v>
       </c>
       <c r="D836" s="11" t="s">
         <v>57</v>
@@ -71753,7 +71744,7 @@
         <v>61</v>
       </c>
       <c r="F836" s="11" t="s">
-        <v>1703</v>
+        <v>1702</v>
       </c>
       <c r="G836" s="12">
         <v>1895</v>
@@ -72368,7 +72359,7 @@
         <v>14</v>
       </c>
       <c r="C844" s="11" t="s">
-        <v>1692</v>
+        <v>1691</v>
       </c>
       <c r="D844" s="11" t="s">
         <v>57</v>
@@ -72377,7 +72368,7 @@
         <v>61</v>
       </c>
       <c r="F844" s="11" t="s">
-        <v>1693</v>
+        <v>1692</v>
       </c>
       <c r="G844" s="12">
         <v>1898</v>
@@ -74552,7 +74543,7 @@
         <v>6</v>
       </c>
       <c r="C872" s="11" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="D872" s="15" t="s">
         <v>80</v>
@@ -74561,7 +74552,7 @@
         <v>26</v>
       </c>
       <c r="F872" s="11" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="G872" s="12">
         <v>1977</v>
@@ -75444,7 +75435,7 @@
   <sheetData>
     <row r="1" spans="1:13" s="16" customFormat="1" ht="21.75" customHeight="1">
       <c r="A1" s="23" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="B1" s="23"/>
       <c r="C1" s="23"/>
@@ -75461,7 +75452,7 @@
     </row>
     <row r="2" spans="1:13" s="16" customFormat="1" ht="21" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="16" customFormat="1" ht="27.75" customHeight="1">
@@ -75475,1409 +75466,545 @@
         <v>27</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>1743</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>1744</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>1745</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>1746</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>1747</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>1748</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>1749</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>1750</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>1751</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>1752</v>
-      </c>
     </row>
     <row r="4" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A4" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>1300</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>1301</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E4" s="26">
-        <v>1819</v>
-      </c>
-      <c r="F4" s="26">
-        <v>1819</v>
-      </c>
-      <c r="G4" s="26">
-        <f t="shared" ref="G4:G37" si="0">IF(OR(E4="",F4=""),"",F4-E4)</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="26">
-        <v>2259</v>
-      </c>
-      <c r="I4" s="26">
-        <v>2259</v>
-      </c>
-      <c r="J4" s="26">
-        <f t="shared" ref="J4:J37" si="1">IF(OR(H4="",I4=""),"",I4-H4)</f>
-        <v>0</v>
-      </c>
-      <c r="K4" s="26">
-        <v>1869</v>
-      </c>
-      <c r="L4" s="26">
-        <v>1819</v>
-      </c>
-      <c r="M4" s="26">
-        <f t="shared" ref="M4:M37" si="2">IF(OR(K4="",L4=""),"",L4-K4)</f>
-        <v>-50</v>
-      </c>
+      <c r="A4" s="19"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
     </row>
     <row r="5" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A5" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>1015</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>1016</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E5" s="26">
-        <v>1839</v>
-      </c>
-      <c r="F5" s="26">
-        <v>1849</v>
-      </c>
-      <c r="G5" s="26">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="H5" s="26">
-        <v>2328</v>
-      </c>
-      <c r="I5" s="26">
-        <v>2328</v>
-      </c>
-      <c r="J5" s="26">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K5" s="26">
-        <v>1829</v>
-      </c>
-      <c r="L5" s="26">
-        <v>1839</v>
-      </c>
-      <c r="M5" s="26">
-        <f t="shared" si="2"/>
-        <v>10</v>
-      </c>
+      <c r="A5" s="19"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
     </row>
     <row r="6" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A6" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>614</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>615</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E6" s="26">
-        <v>1865</v>
-      </c>
-      <c r="F6" s="26">
-        <v>1885</v>
-      </c>
-      <c r="G6" s="26">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="H6" s="26">
-        <v>2225</v>
-      </c>
-      <c r="I6" s="26">
-        <v>2225</v>
-      </c>
-      <c r="J6" s="26">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K6" s="26">
-        <v>1855</v>
-      </c>
-      <c r="L6" s="26">
-        <v>1855</v>
-      </c>
-      <c r="M6" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="A6" s="19"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
     </row>
     <row r="7" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A7" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>1636</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>1637</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E7" s="26">
-        <v>1829</v>
-      </c>
-      <c r="F7" s="26">
-        <v>1819</v>
-      </c>
-      <c r="G7" s="26">
-        <f t="shared" si="0"/>
-        <v>-10</v>
-      </c>
-      <c r="H7" s="26">
-        <v>2285</v>
-      </c>
-      <c r="I7" s="26">
-        <v>2245</v>
-      </c>
-      <c r="J7" s="26">
-        <f t="shared" si="1"/>
-        <v>-40</v>
-      </c>
-      <c r="K7" s="26">
-        <v>1819</v>
-      </c>
-      <c r="L7" s="26">
-        <v>1799</v>
-      </c>
-      <c r="M7" s="26">
-        <f t="shared" si="2"/>
-        <v>-20</v>
-      </c>
+      <c r="A7" s="19"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
     </row>
     <row r="8" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A8" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>1512</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E8" s="26">
-        <v>1834</v>
-      </c>
-      <c r="F8" s="26">
-        <v>1814</v>
-      </c>
-      <c r="G8" s="26">
-        <f t="shared" si="0"/>
-        <v>-20</v>
-      </c>
-      <c r="H8" s="26">
-        <v>2368</v>
-      </c>
-      <c r="I8" s="26">
-        <v>2368</v>
-      </c>
-      <c r="J8" s="26">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K8" s="26">
-        <v>1825</v>
-      </c>
-      <c r="L8" s="26">
-        <v>1825</v>
-      </c>
-      <c r="M8" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="A8" s="19"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
     </row>
     <row r="9" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A9" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>902</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>903</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E9" s="26">
-        <v>1859</v>
-      </c>
-      <c r="F9" s="26">
-        <v>1859</v>
-      </c>
-      <c r="G9" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A9" s="19"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
       <c r="H9" s="26"/>
       <c r="I9" s="26"/>
-      <c r="J9" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="26">
-        <v>1819</v>
-      </c>
-      <c r="L9" s="26">
-        <v>1804</v>
-      </c>
-      <c r="M9" s="26">
-        <f t="shared" si="2"/>
-        <v>-15</v>
-      </c>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
     </row>
     <row r="10" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A10" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>1599</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>1600</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E10" s="26">
-        <v>1819</v>
-      </c>
-      <c r="F10" s="26">
-        <v>1819</v>
-      </c>
-      <c r="G10" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A10" s="19"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
       <c r="H10" s="26"/>
       <c r="I10" s="26"/>
-      <c r="J10" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="26">
-        <v>1809</v>
-      </c>
-      <c r="L10" s="26">
-        <v>1819</v>
-      </c>
-      <c r="M10" s="26">
-        <f t="shared" si="2"/>
-        <v>10</v>
-      </c>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
     </row>
     <row r="11" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A11" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>686</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>687</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E11" s="26">
-        <v>1837</v>
-      </c>
-      <c r="F11" s="26">
-        <v>1837</v>
-      </c>
-      <c r="G11" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A11" s="19"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
       <c r="H11" s="26"/>
       <c r="I11" s="26"/>
-      <c r="J11" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="26">
-        <v>1808</v>
-      </c>
-      <c r="L11" s="26">
-        <v>1793</v>
-      </c>
-      <c r="M11" s="26">
-        <f t="shared" si="2"/>
-        <v>-15</v>
-      </c>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
     </row>
     <row r="12" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A12" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>482</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>483</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E12" s="26">
-        <v>1845</v>
-      </c>
-      <c r="F12" s="26">
-        <v>1845</v>
-      </c>
-      <c r="G12" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A12" s="19"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
       <c r="H12" s="26"/>
       <c r="I12" s="26"/>
-      <c r="J12" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="26">
-        <v>1839</v>
-      </c>
-      <c r="L12" s="26">
-        <v>1824</v>
-      </c>
-      <c r="M12" s="26">
-        <f t="shared" si="2"/>
-        <v>-15</v>
-      </c>
+      <c r="J12" s="26"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="26"/>
+      <c r="M12" s="26"/>
     </row>
     <row r="13" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A13" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>1658</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>1659</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E13" s="26">
-        <v>1899</v>
-      </c>
-      <c r="F13" s="26">
-        <v>1869</v>
-      </c>
-      <c r="G13" s="26">
-        <f t="shared" si="0"/>
-        <v>-30</v>
-      </c>
+      <c r="A13" s="19"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
       <c r="H13" s="26"/>
       <c r="I13" s="26"/>
-      <c r="J13" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="26">
-        <v>1849</v>
-      </c>
-      <c r="L13" s="26">
-        <v>1849</v>
-      </c>
-      <c r="M13" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
+      <c r="L13" s="26"/>
+      <c r="M13" s="26"/>
     </row>
     <row r="14" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A14" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>788</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>789</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E14" s="26">
-        <v>1859</v>
-      </c>
-      <c r="F14" s="26">
-        <v>2199</v>
-      </c>
-      <c r="G14" s="26">
-        <f t="shared" si="0"/>
-        <v>340</v>
-      </c>
+      <c r="A14" s="19"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
       <c r="H14" s="26"/>
       <c r="I14" s="26"/>
-      <c r="J14" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="26">
-        <v>1849</v>
-      </c>
-      <c r="L14" s="26">
-        <v>2199</v>
-      </c>
-      <c r="M14" s="26">
-        <f t="shared" si="2"/>
-        <v>350</v>
-      </c>
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="26"/>
+      <c r="M14" s="26"/>
     </row>
     <row r="15" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A15" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>863</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>864</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E15" s="26">
-        <v>1885</v>
-      </c>
-      <c r="F15" s="26">
-        <v>1885</v>
-      </c>
-      <c r="G15" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A15" s="19"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
       <c r="H15" s="26"/>
       <c r="I15" s="26"/>
-      <c r="J15" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="26">
-        <v>1875</v>
-      </c>
-      <c r="L15" s="26">
-        <v>1845</v>
-      </c>
-      <c r="M15" s="26">
-        <f t="shared" si="2"/>
-        <v>-30</v>
-      </c>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="26"/>
     </row>
     <row r="16" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A16" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="20" t="s">
-        <v>1318</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>1319</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E16" s="26">
-        <v>1887</v>
-      </c>
-      <c r="F16" s="26">
-        <v>1887</v>
-      </c>
-      <c r="G16" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A16" s="19"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
       <c r="H16" s="26"/>
       <c r="I16" s="26"/>
-      <c r="J16" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="26">
-        <v>1853</v>
-      </c>
-      <c r="L16" s="26">
-        <v>1868</v>
-      </c>
-      <c r="M16" s="26">
-        <f t="shared" si="2"/>
-        <v>15</v>
-      </c>
+      <c r="J16" s="26"/>
+      <c r="K16" s="26"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
     </row>
     <row r="17" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A17" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>908</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>909</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E17" s="26">
-        <v>1889</v>
-      </c>
-      <c r="F17" s="26">
-        <v>1889</v>
-      </c>
-      <c r="G17" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A17" s="19"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
       <c r="H17" s="26"/>
       <c r="I17" s="26"/>
-      <c r="J17" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="26">
-        <v>1889</v>
-      </c>
-      <c r="L17" s="26">
-        <v>1879</v>
-      </c>
-      <c r="M17" s="26">
-        <f t="shared" si="2"/>
-        <v>-10</v>
-      </c>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="26"/>
     </row>
     <row r="18" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A18" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="20" t="s">
-        <v>828</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>829</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E18" s="26">
-        <v>1949</v>
-      </c>
-      <c r="F18" s="26">
-        <v>1949</v>
-      </c>
-      <c r="G18" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A18" s="19"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
       <c r="H18" s="26"/>
       <c r="I18" s="26"/>
-      <c r="J18" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="26">
-        <v>2039</v>
-      </c>
-      <c r="L18" s="26">
-        <v>1939</v>
-      </c>
-      <c r="M18" s="26">
-        <f t="shared" si="2"/>
-        <v>-100</v>
-      </c>
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
     </row>
     <row r="19" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A19" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>569</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>571</v>
-      </c>
-      <c r="D19" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E19" s="26">
-        <v>1969</v>
-      </c>
+      <c r="A19" s="19"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="26"/>
       <c r="F19" s="26"/>
-      <c r="G19" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
+      <c r="G19" s="26"/>
       <c r="H19" s="26"/>
       <c r="I19" s="26"/>
-      <c r="J19" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="26">
-        <v>1899</v>
-      </c>
-      <c r="L19" s="26">
-        <v>1899</v>
-      </c>
-      <c r="M19" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="26"/>
     </row>
     <row r="20" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A20" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E20" s="26">
-        <v>1814</v>
-      </c>
-      <c r="F20" s="26">
-        <v>1814</v>
-      </c>
-      <c r="G20" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A20" s="19"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
-      <c r="J20" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="26">
-        <v>1999</v>
-      </c>
-      <c r="L20" s="26">
-        <v>1794</v>
-      </c>
-      <c r="M20" s="26">
-        <f t="shared" si="2"/>
-        <v>-205</v>
-      </c>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
     </row>
     <row r="21" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A21" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>629</v>
-      </c>
-      <c r="C21" s="20" t="s">
-        <v>630</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E21" s="26">
-        <v>1819</v>
-      </c>
-      <c r="F21" s="26">
-        <v>1809</v>
-      </c>
-      <c r="G21" s="26">
-        <f t="shared" si="0"/>
-        <v>-10</v>
-      </c>
+      <c r="A21" s="19"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
       <c r="H21" s="26"/>
       <c r="I21" s="26"/>
-      <c r="J21" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="26">
-        <v>1789</v>
-      </c>
-      <c r="L21" s="26">
-        <v>1789</v>
-      </c>
-      <c r="M21" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="26"/>
+      <c r="M21" s="26"/>
     </row>
     <row r="22" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A22" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>386</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>387</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E22" s="26">
-        <v>1829</v>
-      </c>
-      <c r="F22" s="26">
-        <v>1819</v>
-      </c>
-      <c r="G22" s="26">
-        <f t="shared" si="0"/>
-        <v>-10</v>
-      </c>
+      <c r="A22" s="19"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
       <c r="H22" s="26"/>
       <c r="I22" s="26"/>
-      <c r="J22" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="26">
-        <v>1828</v>
-      </c>
-      <c r="L22" s="26">
-        <v>1818</v>
-      </c>
-      <c r="M22" s="26">
-        <f t="shared" si="2"/>
-        <v>-10</v>
-      </c>
+      <c r="J22" s="26"/>
+      <c r="K22" s="26"/>
+      <c r="L22" s="26"/>
+      <c r="M22" s="26"/>
     </row>
     <row r="23" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A23" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23" s="20" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>1105</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E23" s="26">
-        <v>1838</v>
-      </c>
-      <c r="F23" s="26">
-        <v>1858</v>
-      </c>
-      <c r="G23" s="26">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
+      <c r="A23" s="19"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
       <c r="H23" s="26"/>
       <c r="I23" s="26"/>
-      <c r="J23" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="26">
-        <v>1818</v>
-      </c>
-      <c r="L23" s="26">
-        <v>1838</v>
-      </c>
-      <c r="M23" s="26">
-        <f t="shared" si="2"/>
-        <v>20</v>
-      </c>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="26"/>
+      <c r="M23" s="26"/>
     </row>
     <row r="24" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A24" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" s="20" t="s">
-        <v>1203</v>
-      </c>
-      <c r="C24" s="20" t="s">
-        <v>1204</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E24" s="26">
-        <v>1839</v>
-      </c>
-      <c r="F24" s="26">
-        <v>1829</v>
-      </c>
-      <c r="G24" s="26">
-        <f t="shared" si="0"/>
-        <v>-10</v>
-      </c>
+      <c r="A24" s="19"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
       <c r="H24" s="26"/>
       <c r="I24" s="26"/>
-      <c r="J24" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="26">
-        <v>1828</v>
-      </c>
-      <c r="L24" s="26">
-        <v>1818</v>
-      </c>
-      <c r="M24" s="26">
-        <f t="shared" si="2"/>
-        <v>-10</v>
-      </c>
+      <c r="J24" s="26"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
     </row>
     <row r="25" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A25" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>112</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E25" s="26">
-        <v>1842</v>
-      </c>
-      <c r="F25" s="26">
-        <v>1822</v>
-      </c>
-      <c r="G25" s="26">
-        <f t="shared" si="0"/>
-        <v>-20</v>
-      </c>
+      <c r="A25" s="19"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
       <c r="H25" s="26"/>
       <c r="I25" s="26"/>
-      <c r="J25" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="26">
-        <v>1832</v>
-      </c>
-      <c r="L25" s="26">
-        <v>1802</v>
-      </c>
-      <c r="M25" s="26">
-        <f t="shared" si="2"/>
-        <v>-30</v>
-      </c>
+      <c r="J25" s="26"/>
+      <c r="K25" s="26"/>
+      <c r="L25" s="26"/>
+      <c r="M25" s="26"/>
     </row>
     <row r="26" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A26" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>130</v>
-      </c>
-      <c r="C26" s="20" t="s">
-        <v>131</v>
-      </c>
-      <c r="D26" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E26" s="26">
-        <v>1842</v>
-      </c>
-      <c r="F26" s="26">
-        <v>1824</v>
-      </c>
-      <c r="G26" s="26">
-        <f t="shared" si="0"/>
-        <v>-18</v>
-      </c>
+      <c r="A26" s="19"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
       <c r="H26" s="26"/>
       <c r="I26" s="26"/>
-      <c r="J26" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="26">
-        <v>1842</v>
-      </c>
-      <c r="L26" s="26">
-        <v>1824</v>
-      </c>
-      <c r="M26" s="26">
-        <f t="shared" si="2"/>
-        <v>-18</v>
-      </c>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
+      <c r="L26" s="26"/>
+      <c r="M26" s="26"/>
     </row>
     <row r="27" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A27" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>739</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>740</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E27" s="26">
-        <v>1843</v>
-      </c>
-      <c r="F27" s="26">
-        <v>1843</v>
-      </c>
-      <c r="G27" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A27" s="19"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
       <c r="H27" s="26"/>
       <c r="I27" s="26"/>
-      <c r="J27" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="26">
-        <v>1828</v>
-      </c>
-      <c r="L27" s="26">
-        <v>1823</v>
-      </c>
-      <c r="M27" s="26">
-        <f t="shared" si="2"/>
-        <v>-5</v>
-      </c>
+      <c r="J27" s="26"/>
+      <c r="K27" s="26"/>
+      <c r="L27" s="26"/>
+      <c r="M27" s="26"/>
     </row>
     <row r="28" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A28" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>1207</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>1208</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E28" s="26">
-        <v>1844</v>
-      </c>
-      <c r="F28" s="26">
-        <v>1842</v>
-      </c>
-      <c r="G28" s="26">
-        <f t="shared" si="0"/>
-        <v>-2</v>
-      </c>
+      <c r="A28" s="19"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
       <c r="H28" s="26"/>
       <c r="I28" s="26"/>
-      <c r="J28" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="26">
-        <v>1815</v>
-      </c>
-      <c r="L28" s="26">
-        <v>1825</v>
-      </c>
-      <c r="M28" s="26">
-        <f t="shared" si="2"/>
-        <v>10</v>
-      </c>
+      <c r="J28" s="26"/>
+      <c r="K28" s="26"/>
+      <c r="L28" s="26"/>
+      <c r="M28" s="26"/>
     </row>
     <row r="29" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A29" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B29" s="20" t="s">
-        <v>772</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>773</v>
-      </c>
-      <c r="D29" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E29" s="26">
-        <v>1845</v>
-      </c>
-      <c r="F29" s="26">
-        <v>1825</v>
-      </c>
-      <c r="G29" s="26">
-        <f t="shared" si="0"/>
-        <v>-20</v>
-      </c>
+      <c r="A29" s="19"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
       <c r="H29" s="26"/>
       <c r="I29" s="26"/>
-      <c r="J29" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="26">
-        <v>1815</v>
-      </c>
-      <c r="L29" s="26">
-        <v>1799</v>
-      </c>
-      <c r="M29" s="26">
-        <f t="shared" si="2"/>
-        <v>-16</v>
-      </c>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="26"/>
+      <c r="M29" s="26"/>
     </row>
     <row r="30" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A30" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>459</v>
-      </c>
-      <c r="C30" s="20" t="s">
-        <v>460</v>
-      </c>
-      <c r="D30" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E30" s="26">
-        <v>1870</v>
-      </c>
-      <c r="F30" s="26">
-        <v>1870</v>
-      </c>
-      <c r="G30" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A30" s="19"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
       <c r="H30" s="26"/>
       <c r="I30" s="26"/>
-      <c r="J30" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="26">
-        <v>1900</v>
-      </c>
-      <c r="L30" s="26">
-        <v>1860</v>
-      </c>
-      <c r="M30" s="26">
-        <f t="shared" si="2"/>
-        <v>-40</v>
-      </c>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
     </row>
     <row r="31" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A31" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B31" s="20" t="s">
-        <v>876</v>
-      </c>
-      <c r="C31" s="20" t="s">
-        <v>877</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E31" s="26">
-        <v>1875</v>
-      </c>
-      <c r="F31" s="26">
-        <v>1855</v>
-      </c>
-      <c r="G31" s="26">
-        <f t="shared" si="0"/>
-        <v>-20</v>
-      </c>
+      <c r="A31" s="19"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
       <c r="H31" s="26"/>
       <c r="I31" s="26"/>
-      <c r="J31" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="26">
-        <v>1825</v>
-      </c>
-      <c r="L31" s="26">
-        <v>1825</v>
-      </c>
-      <c r="M31" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
+      <c r="L31" s="26"/>
+      <c r="M31" s="26"/>
     </row>
     <row r="32" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A32" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B32" s="20" t="s">
-        <v>1660</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>1661</v>
-      </c>
-      <c r="D32" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E32" s="26">
-        <v>1889</v>
-      </c>
-      <c r="F32" s="26">
-        <v>1889</v>
-      </c>
-      <c r="G32" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A32" s="19"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
       <c r="H32" s="26"/>
       <c r="I32" s="26"/>
-      <c r="J32" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="26">
-        <v>1824</v>
-      </c>
-      <c r="L32" s="26">
-        <v>1869</v>
-      </c>
-      <c r="M32" s="26">
-        <f t="shared" si="2"/>
-        <v>45</v>
-      </c>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
+      <c r="L32" s="26"/>
+      <c r="M32" s="26"/>
     </row>
     <row r="33" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A33" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B33" s="20" t="s">
-        <v>649</v>
-      </c>
-      <c r="C33" s="20" t="s">
-        <v>650</v>
-      </c>
-      <c r="D33" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E33" s="26">
-        <v>1889</v>
-      </c>
-      <c r="F33" s="26">
-        <v>1889</v>
-      </c>
-      <c r="G33" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A33" s="19"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
       <c r="H33" s="26"/>
       <c r="I33" s="26"/>
-      <c r="J33" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="26">
-        <v>1879</v>
-      </c>
-      <c r="L33" s="26">
-        <v>1859</v>
-      </c>
-      <c r="M33" s="26">
-        <f t="shared" si="2"/>
-        <v>-20</v>
-      </c>
+      <c r="J33" s="26"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="26"/>
+      <c r="M33" s="26"/>
     </row>
     <row r="34" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A34" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>1161</v>
-      </c>
-      <c r="C34" s="20" t="s">
-        <v>1162</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E34" s="26">
-        <v>1895</v>
-      </c>
-      <c r="F34" s="26">
-        <v>1885</v>
-      </c>
-      <c r="G34" s="26">
-        <f t="shared" si="0"/>
-        <v>-10</v>
-      </c>
+      <c r="A34" s="19"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
       <c r="H34" s="26"/>
       <c r="I34" s="26"/>
-      <c r="J34" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="26">
-        <v>1875</v>
-      </c>
-      <c r="L34" s="26">
-        <v>1875</v>
-      </c>
-      <c r="M34" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="26"/>
+      <c r="M34" s="26"/>
     </row>
     <row r="35" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A35" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>1125</v>
-      </c>
-      <c r="C35" s="20" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E35" s="26">
-        <v>1909</v>
-      </c>
-      <c r="F35" s="26">
-        <v>1909</v>
-      </c>
-      <c r="G35" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A35" s="19"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
+      <c r="G35" s="26"/>
       <c r="H35" s="26"/>
       <c r="I35" s="26"/>
-      <c r="J35" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="26">
-        <v>1899</v>
-      </c>
-      <c r="L35" s="26">
-        <v>1860</v>
-      </c>
-      <c r="M35" s="26">
-        <f t="shared" si="2"/>
-        <v>-39</v>
-      </c>
+      <c r="J35" s="26"/>
+      <c r="K35" s="26"/>
+      <c r="L35" s="26"/>
+      <c r="M35" s="26"/>
     </row>
     <row r="36" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A36" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B36" s="20" t="s">
-        <v>1117</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>1118</v>
-      </c>
-      <c r="D36" s="20" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E36" s="26">
-        <v>1949</v>
-      </c>
-      <c r="F36" s="26">
-        <v>1899</v>
-      </c>
-      <c r="G36" s="26">
-        <f t="shared" si="0"/>
-        <v>-50</v>
-      </c>
+      <c r="A36" s="19"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
       <c r="H36" s="26"/>
       <c r="I36" s="26"/>
-      <c r="J36" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="26">
-        <v>1929</v>
-      </c>
-      <c r="L36" s="26">
-        <v>1929</v>
-      </c>
-      <c r="M36" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="J36" s="26"/>
+      <c r="K36" s="26"/>
+      <c r="L36" s="26"/>
+      <c r="M36" s="26"/>
     </row>
     <row r="37" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A37" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B37" s="20" t="s">
-        <v>1678</v>
-      </c>
-      <c r="C37" s="20" t="s">
-        <v>1680</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>1766</v>
-      </c>
-      <c r="E37" s="26">
-        <v>1824</v>
-      </c>
+      <c r="A37" s="19"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="26"/>
       <c r="F37" s="26"/>
-      <c r="G37" s="26" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
+      <c r="G37" s="26"/>
       <c r="H37" s="26"/>
       <c r="I37" s="26"/>
-      <c r="J37" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="26">
-        <v>1813</v>
-      </c>
+      <c r="J37" s="26"/>
+      <c r="K37" s="26"/>
       <c r="L37" s="26"/>
-      <c r="M37" s="26" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
+      <c r="M37" s="26"/>
     </row>
     <row r="38" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
       <c r="A38" s="19"/>
@@ -79974,7 +79101,7 @@
     <mergeCell ref="A1:M1"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
-  <conditionalFormatting sqref="G4:G37">
+  <conditionalFormatting sqref="G4">
     <cfRule type="cellIs" dxfId="5" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
@@ -79982,7 +79109,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J4:J37">
+  <conditionalFormatting sqref="J4">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
@@ -79990,7 +79117,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M4:M37">
+  <conditionalFormatting sqref="M4">
     <cfRule type="cellIs" dxfId="1" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Refresh verified fuel workbook after additional candidate validation
Preserve the canonical formula buffer and scan-boundary optimization in
6f073342. Refresh from live Opinet using that actual release binary with
--verify, and independently check ZIP integrity. No product code or
verification workflow changes are included in this commit.

Source acquired 2026-09-06 05:51-05:52 UTC. Retain 869 stations in seven
regions; this refresh found zero station changes, additions or closures.
Workbook SHA-256:
222126153c1464b4977ccce7e7b26ab48a685d450ea09451f9f42b777f734c62

Evidence: Actions 34014561464 and final receipt 34015294367.
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4706" uniqueCount="1766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4702" uniqueCount="1765">
   <si>
     <t>유류비 계산(혼유, 지역화폐 등)</t>
   </si>
@@ -5383,9 +5383,6 @@
   </si>
   <si>
     <t>충북 청주시 청원구 직지대로 830</t>
-  </si>
-  <si>
-    <t>가격변동</t>
   </si>
   <si>
     <t>세종시 부강면 시목부강로 423</t>
@@ -49609,7 +49606,7 @@
         <v>26</v>
       </c>
       <c r="F552" s="11" t="s">
-        <v>1764</v>
+        <v>1763</v>
       </c>
       <c r="G552" s="12">
         <v>1824</v>
@@ -75540,7 +75537,7 @@
     </row>
     <row r="2" spans="1:13" s="16" customFormat="1" ht="21" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>1765</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="16" customFormat="1" ht="27.75" customHeight="1">
@@ -75585,44 +75582,19 @@
       </c>
     </row>
     <row r="4" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A4" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>1193</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>1194</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>1763</v>
-      </c>
-      <c r="E4" s="26">
-        <v>1838</v>
-      </c>
-      <c r="F4" s="26">
-        <v>1838</v>
-      </c>
-      <c r="G4" s="26">
-        <f>IF(OR(E4="",F4=""),"",F4-E4)</f>
-        <v>0</v>
-      </c>
+      <c r="A4" s="19"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
       <c r="H4" s="26"/>
       <c r="I4" s="26"/>
-      <c r="J4" s="26" t="str">
-        <f>IF(OR(H4="",I4=""),"",I4-H4)</f>
-        <v/>
-      </c>
-      <c r="K4" s="26">
-        <v>1848</v>
-      </c>
-      <c r="L4" s="26">
-        <v>1818</v>
-      </c>
-      <c r="M4" s="26">
-        <f>IF(OR(K4="",L4=""),"",L4-K4)</f>
-        <v>-30</v>
-      </c>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
     </row>
     <row r="5" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
       <c r="A5" s="19"/>

</xml_diff>

<commit_message>
Assemble replacement formulas with one allocation
Preserve formula XML and cached values while removing an intermediate string. Fixed-corpus release measurements show lower time and allocation counts; workbook bytes match the baseline. Validated with Rust 1.98.1 host and six-target Clippy, allocation failure and corrupted-input probes, and verified workbook refresh.
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4685" uniqueCount="1758">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4681" uniqueCount="1757">
   <si>
     <t>유류비 계산(혼유, 지역화폐 등)</t>
   </si>
@@ -5362,9 +5362,6 @@
   </si>
   <si>
     <t>세종시 부강면 시목부강로 423</t>
-  </si>
-  <si>
-    <t>가격변동</t>
   </si>
   <si>
     <t>현행화 일자: 2026-09-09</t>
@@ -75198,7 +75195,7 @@
     </row>
     <row r="2" spans="1:13" s="16" customFormat="1" ht="21" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>1757</v>
+        <v>1756</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="16" customFormat="1" ht="27.75" customHeight="1">
@@ -75243,44 +75240,19 @@
       </c>
     </row>
     <row r="4" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A4" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>910</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>911</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>1756</v>
-      </c>
-      <c r="E4" s="26">
-        <v>1814</v>
-      </c>
-      <c r="F4" s="26">
-        <v>1799</v>
-      </c>
-      <c r="G4" s="26">
-        <f>IF(OR(E4="",F4=""),"",F4-E4)</f>
-        <v>-15</v>
-      </c>
+      <c r="A4" s="19"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
       <c r="H4" s="26"/>
       <c r="I4" s="26"/>
-      <c r="J4" s="26" t="str">
-        <f>IF(OR(H4="",I4=""),"",I4-H4)</f>
-        <v/>
-      </c>
-      <c r="K4" s="26">
-        <v>1794</v>
-      </c>
-      <c r="L4" s="26">
-        <v>1794</v>
-      </c>
-      <c r="M4" s="26">
-        <f>IF(OR(K4="",L4=""),"",L4-K4)</f>
-        <v>0</v>
-      </c>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
     </row>
     <row r="5" spans="1:13" s="16" customFormat="1" ht="25.5" customHeight="1">
       <c r="A5" s="19"/>

</xml_diff>